<commit_message>
Agregar control de reglas de calidad y actualizar completitud
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FORMATO_MVP_diligenciado/FORMATO_MVP_diligenciado.xlsx
+++ b/FORMATO_MVP_diligenciado/FORMATO_MVP_diligenciado.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30318"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30317"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="37" documentId="11_38300255FD6531415D2E1AB2F1D62E0D8F30DD3A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F706C5CF-C03B-45B8-8259-8A7B8D357405}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="11_38300255FD6531415D2E1AB2F1D62E0D8F30DD3A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A24E711-2C1B-4270-9090-892FD9C84CCA}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Instrucciones" sheetId="1" r:id="rId1"/>
-    <sheet name="HU" sheetId="2" r:id="rId2"/>
+    <sheet name="HU" sheetId="2" r:id="rId1"/>
+    <sheet name="Instrucciones" sheetId="1" r:id="rId2"/>
     <sheet name="Diccionario_Datos" sheetId="3" r:id="rId3"/>
     <sheet name="Formato KPI" sheetId="4" r:id="rId4"/>
     <sheet name="Formato_reglas_calidad" sheetId="5" r:id="rId5"/>
@@ -114,6 +114,102 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="864" uniqueCount="426">
   <si>
+    <t xml:space="preserve"> FORMATO DEFINICIÓN DE ALCANCE PARA DESARROLLO DE PRODUCTOS DE DATOS</t>
+  </si>
+  <si>
+    <t>Sección</t>
+  </si>
+  <si>
+    <t>Detalle</t>
+  </si>
+  <si>
+    <t>Contexto y objetivo de producto</t>
+  </si>
+  <si>
+    <t>Se detectó una diferencia de más de 3 millones de pesos en la prima entre el DWH y el CDP para ciertos meses, aunque la cantidad de pólizas sí coincide entre ambos sistemas. Como respuesta, Gobierno de Datos necesita un control de completitud que avise, ANTES del cierre contable (~día 10 de cada mes), si a alguna cuenta contable le está faltando información en el DWH.</t>
+  </si>
+  <si>
+    <t>Historia de Usuario</t>
+  </si>
+  <si>
+    <t>Cómo?</t>
+  </si>
+  <si>
+    <t>Mediante un control automático (script SQL: control_completitud_cuentas.sql) que verifica que VALOR_RESERVA_CONTABLE tenga valor para cada cuenta + libro + periodo en el DWH</t>
+  </si>
+  <si>
+    <t>Quien?</t>
+  </si>
+  <si>
+    <t>Analista de Gobierno de Datos</t>
+  </si>
+  <si>
+    <t>Para qué?</t>
+  </si>
+  <si>
+    <t>para alertar al dueño de la tabla los días 8-9 de cada mes, antes del cierre contable del día 10, y evitar que el reporte oficial salga con información incompleta</t>
+  </si>
+  <si>
+    <t>Criterios de Aceptación</t>
+  </si>
+  <si>
+    <t>Campos de salida: fuente, cuenta, libro, periodo_contable_analisis, total_registros, con_valor, sin_valor, pct_completitud, semaforo.</t>
+  </si>
+  <si>
+    <t>Fuentes de datos (DWH SQL Server, base Liberty, esquema RESERVAS): DIRECTA_RESERVA_INTERFAZ, CEDIDAS_RESERVA_INTERFAZ, CEDIDAS_RESERVA_INTERFAZ_IAXIS, CEDIDAS_TERREMOTO_RESERVA_INTERFAZ.</t>
+  </si>
+  <si>
+    <t>Formato de salida: tabla resumen tipo semáforo (COMPLETO / ALERTA), ordenada con las ALERTAs primero.</t>
+  </si>
+  <si>
+    <t>Periodicidad: mensual, días 8-9, antes del proceso oficial de cierre (~día 10). Periodo parametrizable vía @PERIODO en formato AAAAMM.</t>
+  </si>
+  <si>
+    <t>Exclusiones: Incurrido, Salvamentos, Recobros e IVA AG (cubierto por el filtro Libro &lt;&gt; 'AG'); hay 2 cuentas adicionales excluidas pendientes de confirmar con Andrey.</t>
+  </si>
+  <si>
+    <t>El control valida únicamente la existencia del dato (no nulo); no valida la razonabilidad del valor.</t>
+  </si>
+  <si>
+    <t>Tipos de Producto (Entregables)</t>
+  </si>
+  <si>
+    <t>Script SQL: control_completitud_cuentas.sql (parámetro @PERIODO en formato AAAAMM).</t>
+  </si>
+  <si>
+    <t>Tabla resumen: una fila por fuente + cuenta + libro + periodo, con porcentaje de completitud y semáforo.</t>
+  </si>
+  <si>
+    <t>Tablero HTML de completitud: notebooks/dashboard_completitud.html (generado desde notebooks/tablero_completitud.ipynb).</t>
+  </si>
+  <si>
+    <t>Documentación: README.md, 'Hallazgos y Estado del Proyecto.md' y OriginProcessql/EXPLICACION_SCRIPTS.md.</t>
+  </si>
+  <si>
+    <t>Restricciones</t>
+  </si>
+  <si>
+    <t>Solo valida que el dato exista (no nulo); la validación de razonabilidad / valores atípicos es la Fase 2, que aún no ha iniciado.</t>
+  </si>
+  <si>
+    <t>El entregable llega hasta el semáforo (COMPLETO/ALERTA); las alertas automáticas las construye el equipo de Andrey por separado.</t>
+  </si>
+  <si>
+    <t>No replica la lógica compleja de los procesos de producción (corretaje/cocorretaje, tomador, intermediarios) — es intencionalmente simple.</t>
+  </si>
+  <si>
+    <t>Valor para el Negocio</t>
+  </si>
+  <si>
+    <t>Detectar antes del cierre mensual las cuentas contables con información incompleta en el DWH, evitando que el reporte oficial salga con errores. Es el prototipo que luego se replicará para el módulo 'canal no tradicional' y convive con otros controles del equipo (ej. cocorretaje en CDP).</t>
+  </si>
+  <si>
+    <t>Validación</t>
+  </si>
+  <si>
+    <t>Responsable de la validación: Andrey (líder del tema en Gobierno de Datos). El script está construido pero aún no se ha probado contra un mes cerrado con datos completos; fecha de validación pendiente.</t>
+  </si>
+  <si>
     <t>Instrucciones de llenado de campos</t>
   </si>
   <si>
@@ -123,25 +219,16 @@
     <t>FORMATO DE FICHA</t>
   </si>
   <si>
-    <t>Sección</t>
-  </si>
-  <si>
     <t>Descripcion</t>
   </si>
   <si>
     <t>Ejemplos:</t>
   </si>
   <si>
-    <t>Contexto y objetivo de producto</t>
-  </si>
-  <si>
     <t>Explica la necesidad del área solicitante y el propósito principal del producto de datos. Debe describir de forma general qué problema se busca resolver o qué información se requiere consolidar, así como el objetivo de negocio que se pretende alcanzar con el producto.</t>
   </si>
   <si>
     <t>El área de ventas requiere un tablero que consolide la información de facturación y clientes para monitorear el desempeño comercial en tiempo real y soportar la toma de decisiones.</t>
-  </si>
-  <si>
-    <t>Historia de Usuario</t>
   </si>
   <si>
     <r>
@@ -254,9 +341,6 @@
     </r>
   </si>
   <si>
-    <t>Criterios de Aceptación</t>
-  </si>
-  <si>
     <t>Conjunto de condiciones que deben cumplirse para considerar el producto de datos como terminado y aceptado. Incluyen los campos requeridos, fuentes autorizadas, formatos de salida, periodicidad, reglas de exclusión y cualquier requisito funcional mínimo que asegure que el producto cumple su propósito.</t>
   </si>
   <si>
@@ -312,9 +396,6 @@
   </si>
   <si>
     <t>- Exclusiones: no incluir filtros dinámicos ni gráficos adicionales fuera de los KPIs definidos.</t>
-  </si>
-  <si>
-    <t>Tipos de Producto (Entregables)</t>
   </si>
   <si>
     <t>Lista de los artefactos que se entregarán como resultado del desarrollo del producto de datos. Incluye tableros, tablas, KPIs, modelos de datos o cualquier salida generada que forme parte del entregable final. Cada elemento debe describir de manera general qué representa y cómo aporta al uso del producto.</t>
@@ -473,9 +554,6 @@
     </r>
   </si>
   <si>
-    <t>Restricciones</t>
-  </si>
-  <si>
     <t>Condiciones o limitaciones que deben respetarse durante el desarrollo y uso del producto de datos. Incluyen restricciones sobre alcances no permitidos, campos autorizados, formatos establecidos, fuentes válidas y cualquier regla que limite modificaciones o ampliaciones fuera del alcance definido.</t>
   </si>
   <si>
@@ -488,16 +566,10 @@
     <t>- No se aceptan modificaciones en el formato acordado.</t>
   </si>
   <si>
-    <t>Valor para el Negocio</t>
-  </si>
-  <si>
     <t>Define los beneficios que el producto de datos aporta al área usuaria. Describe cómo mejora la toma de decisiones, optimiza procesos, genera eficiencia o incrementa visibilidad sobre la operación. Debe expresar el impacto directo del producto en el negocio sin detallar aspectos técnicos.</t>
   </si>
   <si>
     <t>El tablero permitirá al área de ventas monitorear el desempeño comercial, identificar clientes activos e inactivos y tomar decisiones basadas en datos confiables y estandarizados.</t>
-  </si>
-  <si>
-    <t>Validación</t>
   </si>
   <si>
     <t>Registra quién aprueba formalmente el producto de datos antes de su entrega. Incluye los roles responsables de validar el resultado (negocio y datos) y la fecha en que se confirma que el producto cumple con los requisitos definidos.</t>
@@ -1391,78 +1463,6 @@
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve"> FORMATO DEFINICIÓN DE ALCANCE PARA DESARROLLO DE PRODUCTOS DE DATOS</t>
-  </si>
-  <si>
-    <t>Detalle</t>
-  </si>
-  <si>
-    <t>Se detectó una diferencia de más de 3 millones de pesos en la prima entre el DWH y el CDP para ciertos meses, aunque la cantidad de pólizas sí coincide entre ambos sistemas. Como respuesta, Gobierno de Datos necesita un control de completitud que avise, ANTES del cierre contable (~día 10 de cada mes), si a alguna cuenta contable le está faltando información en el DWH.</t>
-  </si>
-  <si>
-    <t>Cómo?</t>
-  </si>
-  <si>
-    <t>Mediante un control automático (script SQL: control_completitud_cuentas.sql) que verifica que VALOR_RESERVA_CONTABLE tenga valor para cada cuenta + libro + periodo en el DWH</t>
-  </si>
-  <si>
-    <t>Quien?</t>
-  </si>
-  <si>
-    <t>Analista de Gobierno de Datos</t>
-  </si>
-  <si>
-    <t>Para qué?</t>
-  </si>
-  <si>
-    <t>para alertar al dueño de la tabla los días 8-9 de cada mes, antes del cierre contable del día 10, y evitar que el reporte oficial salga con información incompleta</t>
-  </si>
-  <si>
-    <t>Campos de salida: fuente, cuenta, libro, periodo_contable_analisis, total_registros, con_valor, sin_valor, pct_completitud, semaforo.</t>
-  </si>
-  <si>
-    <t>Fuentes de datos (DWH SQL Server, base Liberty, esquema RESERVAS): DIRECTA_RESERVA_INTERFAZ, CEDIDAS_RESERVA_INTERFAZ, CEDIDAS_RESERVA_INTERFAZ_IAXIS, CEDIDAS_TERREMOTO_RESERVA_INTERFAZ.</t>
-  </si>
-  <si>
-    <t>Formato de salida: tabla resumen tipo semáforo (COMPLETO / ALERTA), ordenada con las ALERTAs primero.</t>
-  </si>
-  <si>
-    <t>Periodicidad: mensual, días 8-9, antes del proceso oficial de cierre (~día 10). Periodo parametrizable vía @PERIODO en formato AAAAMM.</t>
-  </si>
-  <si>
-    <t>Exclusiones: Incurrido, Salvamentos, Recobros e IVA AG (cubierto por el filtro Libro &lt;&gt; 'AG'); hay 2 cuentas adicionales excluidas pendientes de confirmar con Andrey.</t>
-  </si>
-  <si>
-    <t>El control valida únicamente la existencia del dato (no nulo); no valida la razonabilidad del valor.</t>
-  </si>
-  <si>
-    <t>Script SQL: control_completitud_cuentas.sql (parámetro @PERIODO en formato AAAAMM).</t>
-  </si>
-  <si>
-    <t>Tabla resumen: una fila por fuente + cuenta + libro + periodo, con porcentaje de completitud y semáforo.</t>
-  </si>
-  <si>
-    <t>Tablero HTML de completitud: notebooks/dashboard_completitud.html (generado desde notebooks/tablero_completitud.ipynb).</t>
-  </si>
-  <si>
-    <t>Documentación: README.md, 'Hallazgos y Estado del Proyecto.md' y OriginProcessql/EXPLICACION_SCRIPTS.md.</t>
-  </si>
-  <si>
-    <t>Solo valida que el dato exista (no nulo); la validación de razonabilidad / valores atípicos es la Fase 2, que aún no ha iniciado.</t>
-  </si>
-  <si>
-    <t>El entregable llega hasta el semáforo (COMPLETO/ALERTA); las alertas automáticas las construye el equipo de Andrey por separado.</t>
-  </si>
-  <si>
-    <t>No replica la lógica compleja de los procesos de producción (corretaje/cocorretaje, tomador, intermediarios) — es intencionalmente simple.</t>
-  </si>
-  <si>
-    <t>Detectar antes del cierre mensual las cuentas contables con información incompleta en el DWH, evitando que el reporte oficial salga con errores. Es el prototipo que luego se replicará para el módulo 'canal no tradicional' y convive con otros controles del equipo (ej. cocorretaje en CDP).</t>
-  </si>
-  <si>
-    <t>Responsable de la validación: Andrey (líder del tema en Gobierno de Datos). El script está construido pero aún no se ha probado contra un mes cerrado con datos completos; fecha de validación pendiente.</t>
   </si>
   <si>
     <t>Tipo de tabla origen</t>
@@ -2378,7 +2378,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2584,6 +2584,15 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2591,21 +2600,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2616,6 +2610,9 @@
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2629,14 +2626,14 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2650,6 +2647,9 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2658,6 +2658,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
@@ -3086,6 +3089,204 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:C29"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
+  <cols>
+    <col min="1" max="1" width="18.5703125" customWidth="1"/>
+    <col min="2" max="2" width="86.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="101" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="105"/>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="105"/>
+      <c r="B2" s="105"/>
+    </row>
+    <row r="4" spans="1:3" ht="15" customHeight="1" thickBot="1"/>
+    <row r="5" spans="1:3" ht="15.6" customHeight="1" thickBot="1">
+      <c r="A5" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="126" customHeight="1" thickBot="1">
+      <c r="A6" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15" customHeight="1">
+      <c r="A7" s="102" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15" customHeight="1">
+      <c r="A8" s="106"/>
+      <c r="B8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15.6" customHeight="1" thickBot="1">
+      <c r="A9" s="107"/>
+      <c r="B9" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="30.75">
+      <c r="A10" s="102" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="61.5">
+      <c r="A11" s="106"/>
+      <c r="B11" s="8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="30.75">
+      <c r="A12" s="106"/>
+      <c r="B12" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="30.75">
+      <c r="A13" s="106"/>
+      <c r="B13" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="30.75">
+      <c r="A14" s="106"/>
+      <c r="B14" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="30.75" thickBot="1">
+      <c r="A15" s="107"/>
+      <c r="B15" s="9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="30.75">
+      <c r="A16" s="102" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="30.75">
+      <c r="A17" s="106"/>
+      <c r="B17" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="30.75">
+      <c r="A18" s="106"/>
+      <c r="B18" s="8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="30.75">
+      <c r="A19" s="106"/>
+      <c r="B19" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.6" customHeight="1">
+      <c r="A20" s="106"/>
+      <c r="B20" s="8"/>
+    </row>
+    <row r="21" spans="1:2" ht="15.6" customHeight="1">
+      <c r="A21" s="106"/>
+      <c r="B21" s="8"/>
+    </row>
+    <row r="22" spans="1:2" ht="15.95" customHeight="1" thickBot="1">
+      <c r="A22" s="107"/>
+      <c r="B22" s="9"/>
+    </row>
+    <row r="23" spans="1:2" ht="30.75">
+      <c r="A23" s="102" t="s">
+        <v>24</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="30.75">
+      <c r="A24" s="106"/>
+      <c r="B24" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="30.75" thickBot="1">
+      <c r="A25" s="107"/>
+      <c r="B25" s="9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="30.6" customHeight="1" thickBot="1">
+      <c r="A26" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="15.6" customHeight="1">
+      <c r="A27" s="102" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="15.6" customHeight="1">
+      <c r="A28" s="106"/>
+      <c r="B28" s="8"/>
+    </row>
+    <row r="29" spans="1:2" ht="15.95" customHeight="1" thickBot="1">
+      <c r="A29" s="107"/>
+      <c r="B29" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:B2"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="A16:A22"/>
+    <mergeCell ref="A10:A15"/>
+    <mergeCell ref="A23:A25"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T286"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
@@ -3097,10 +3298,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A1" s="93" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="93"/>
+      <c r="A1" s="92" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="92"/>
       <c r="C1" s="27"/>
       <c r="D1" s="27"/>
       <c r="E1" s="27"/>
@@ -3165,10 +3366,10 @@
       <c r="T3" s="27"/>
     </row>
     <row r="4" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A4" s="97" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="97"/>
+      <c r="A4" s="96" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="96"/>
       <c r="C4" s="28"/>
       <c r="D4" s="27"/>
       <c r="E4" s="27"/>
@@ -3212,7 +3413,7 @@
     </row>
     <row r="6" spans="1:20" ht="15.95" customHeight="1">
       <c r="A6" s="29" t="s">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="B6" s="28"/>
       <c r="C6" s="28"/>
@@ -3236,13 +3437,13 @@
     </row>
     <row r="7" spans="1:20" ht="15.95" customHeight="1">
       <c r="A7" s="30" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B7" s="31" t="s">
-        <v>4</v>
+        <v>35</v>
       </c>
       <c r="C7" s="32" t="s">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="D7" s="27"/>
       <c r="E7" s="27"/>
@@ -3264,13 +3465,13 @@
     </row>
     <row r="8" spans="1:20" ht="74.099999999999994" customHeight="1">
       <c r="A8" s="30" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="C8" s="34" t="s">
-        <v>8</v>
+        <v>38</v>
       </c>
       <c r="D8" s="27"/>
       <c r="E8" s="27"/>
@@ -3291,14 +3492,14 @@
       <c r="T8" s="27"/>
     </row>
     <row r="9" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A9" s="82" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="98" t="s">
-        <v>10</v>
+      <c r="A9" s="93" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="97" t="s">
+        <v>39</v>
       </c>
       <c r="C9" s="35" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="D9" s="27"/>
       <c r="E9" s="27"/>
@@ -3319,10 +3520,10 @@
       <c r="T9" s="27"/>
     </row>
     <row r="10" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A10" s="83"/>
-      <c r="B10" s="99"/>
+      <c r="A10" s="94"/>
+      <c r="B10" s="98"/>
       <c r="C10" s="36" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="D10" s="27"/>
       <c r="E10" s="27"/>
@@ -3343,10 +3544,10 @@
       <c r="T10" s="27"/>
     </row>
     <row r="11" spans="1:20" ht="21" customHeight="1">
-      <c r="A11" s="84"/>
-      <c r="B11" s="100"/>
+      <c r="A11" s="95"/>
+      <c r="B11" s="99"/>
       <c r="C11" s="37" t="s">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="D11" s="27"/>
       <c r="E11" s="27"/>
@@ -3367,14 +3568,14 @@
       <c r="T11" s="27"/>
     </row>
     <row r="12" spans="1:20" ht="30.95" customHeight="1">
-      <c r="A12" s="82" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" s="94" t="s">
-        <v>15</v>
+      <c r="A12" s="93" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="79" t="s">
+        <v>43</v>
       </c>
       <c r="C12" s="38" t="s">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="D12" s="27"/>
       <c r="E12" s="27"/>
@@ -3395,10 +3596,10 @@
       <c r="T12" s="27"/>
     </row>
     <row r="13" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A13" s="83"/>
-      <c r="B13" s="95"/>
+      <c r="A13" s="94"/>
+      <c r="B13" s="80"/>
       <c r="C13" s="39" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="D13" s="27"/>
       <c r="E13" s="27"/>
@@ -3419,10 +3620,10 @@
       <c r="T13" s="27"/>
     </row>
     <row r="14" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A14" s="83"/>
-      <c r="B14" s="95"/>
+      <c r="A14" s="94"/>
+      <c r="B14" s="80"/>
       <c r="C14" s="39" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="D14" s="27"/>
       <c r="E14" s="27"/>
@@ -3443,10 +3644,10 @@
       <c r="T14" s="27"/>
     </row>
     <row r="15" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A15" s="83"/>
-      <c r="B15" s="95"/>
+      <c r="A15" s="94"/>
+      <c r="B15" s="80"/>
       <c r="C15" s="39" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="D15" s="27"/>
       <c r="E15" s="27"/>
@@ -3467,10 +3668,10 @@
       <c r="T15" s="27"/>
     </row>
     <row r="16" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A16" s="83"/>
-      <c r="B16" s="95"/>
+      <c r="A16" s="94"/>
+      <c r="B16" s="80"/>
       <c r="C16" s="39" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="D16" s="27"/>
       <c r="E16" s="27"/>
@@ -3491,10 +3692,10 @@
       <c r="T16" s="27"/>
     </row>
     <row r="17" spans="1:20" ht="32.1" customHeight="1">
-      <c r="A17" s="84"/>
-      <c r="B17" s="96"/>
+      <c r="A17" s="95"/>
+      <c r="B17" s="81"/>
       <c r="C17" s="40" t="s">
-        <v>21</v>
+        <v>49</v>
       </c>
       <c r="D17" s="27"/>
       <c r="E17" s="27"/>
@@ -3515,14 +3716,14 @@
       <c r="T17" s="27"/>
     </row>
     <row r="18" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A18" s="82" t="s">
-        <v>22</v>
-      </c>
-      <c r="B18" s="94" t="s">
-        <v>23</v>
+      <c r="A18" s="93" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="79" t="s">
+        <v>50</v>
       </c>
       <c r="C18" s="38" t="s">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="D18" s="27"/>
       <c r="E18" s="27"/>
@@ -3543,10 +3744,10 @@
       <c r="T18" s="27"/>
     </row>
     <row r="19" spans="1:20" ht="35.1" customHeight="1">
-      <c r="A19" s="83"/>
-      <c r="B19" s="95"/>
+      <c r="A19" s="94"/>
+      <c r="B19" s="80"/>
       <c r="C19" s="39" t="s">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="D19" s="27"/>
       <c r="E19" s="27"/>
@@ -3567,10 +3768,10 @@
       <c r="T19" s="27"/>
     </row>
     <row r="20" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A20" s="83"/>
-      <c r="B20" s="95"/>
+      <c r="A20" s="94"/>
+      <c r="B20" s="80"/>
       <c r="C20" s="39" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="D20" s="27"/>
       <c r="E20" s="27"/>
@@ -3591,10 +3792,10 @@
       <c r="T20" s="27"/>
     </row>
     <row r="21" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A21" s="83"/>
-      <c r="B21" s="95"/>
+      <c r="A21" s="94"/>
+      <c r="B21" s="80"/>
       <c r="C21" s="39" t="s">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="D21" s="27"/>
       <c r="E21" s="27"/>
@@ -3615,10 +3816,10 @@
       <c r="T21" s="27"/>
     </row>
     <row r="22" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A22" s="83"/>
-      <c r="B22" s="95"/>
+      <c r="A22" s="94"/>
+      <c r="B22" s="80"/>
       <c r="C22" s="39" t="s">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="D22" s="27"/>
       <c r="E22" s="27"/>
@@ -3639,10 +3840,10 @@
       <c r="T22" s="27"/>
     </row>
     <row r="23" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A23" s="83"/>
-      <c r="B23" s="95"/>
+      <c r="A23" s="94"/>
+      <c r="B23" s="80"/>
       <c r="C23" s="39" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="D23" s="27"/>
       <c r="E23" s="27"/>
@@ -3663,10 +3864,10 @@
       <c r="T23" s="27"/>
     </row>
     <row r="24" spans="1:20" ht="31.5" customHeight="1">
-      <c r="A24" s="84"/>
-      <c r="B24" s="96"/>
+      <c r="A24" s="95"/>
+      <c r="B24" s="81"/>
       <c r="C24" s="40" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="D24" s="27"/>
       <c r="E24" s="27"/>
@@ -3687,14 +3888,14 @@
       <c r="T24" s="27"/>
     </row>
     <row r="25" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A25" s="82" t="s">
-        <v>31</v>
-      </c>
-      <c r="B25" s="94" t="s">
-        <v>32</v>
+      <c r="A25" s="93" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" s="79" t="s">
+        <v>58</v>
       </c>
       <c r="C25" s="38" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="D25" s="27"/>
       <c r="E25" s="27"/>
@@ -3715,10 +3916,10 @@
       <c r="T25" s="27"/>
     </row>
     <row r="26" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A26" s="83"/>
-      <c r="B26" s="95"/>
+      <c r="A26" s="94"/>
+      <c r="B26" s="80"/>
       <c r="C26" s="39" t="s">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="D26" s="27"/>
       <c r="E26" s="27"/>
@@ -3739,10 +3940,10 @@
       <c r="T26" s="27"/>
     </row>
     <row r="27" spans="1:20" ht="15.95" customHeight="1">
-      <c r="A27" s="84"/>
-      <c r="B27" s="96"/>
+      <c r="A27" s="95"/>
+      <c r="B27" s="81"/>
       <c r="C27" s="40" t="s">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="D27" s="27"/>
       <c r="E27" s="27"/>
@@ -3764,13 +3965,13 @@
     </row>
     <row r="28" spans="1:20" ht="62.45" customHeight="1">
       <c r="A28" s="30" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="B28" s="41" t="s">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="C28" s="42" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="D28" s="27"/>
       <c r="E28" s="27"/>
@@ -3791,14 +3992,14 @@
       <c r="T28" s="27"/>
     </row>
     <row r="29" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A29" s="82" t="s">
-        <v>39</v>
-      </c>
-      <c r="B29" s="94" t="s">
-        <v>40</v>
+      <c r="A29" s="93" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" s="79" t="s">
+        <v>64</v>
       </c>
       <c r="C29" s="38" t="s">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="D29" s="27"/>
       <c r="E29" s="27"/>
@@ -3819,10 +4020,10 @@
       <c r="T29" s="27"/>
     </row>
     <row r="30" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A30" s="83"/>
-      <c r="B30" s="95"/>
+      <c r="A30" s="94"/>
+      <c r="B30" s="80"/>
       <c r="C30" s="39" t="s">
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="D30" s="27"/>
       <c r="E30" s="27"/>
@@ -3843,10 +4044,10 @@
       <c r="T30" s="27"/>
     </row>
     <row r="31" spans="1:20" ht="15.95" customHeight="1">
-      <c r="A31" s="84"/>
-      <c r="B31" s="96"/>
+      <c r="A31" s="95"/>
+      <c r="B31" s="81"/>
       <c r="C31" s="43" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="D31" s="27"/>
       <c r="E31" s="27"/>
@@ -3955,10 +4156,10 @@
       <c r="T35" s="27"/>
     </row>
     <row r="36" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A36" s="85" t="s">
-        <v>44</v>
-      </c>
-      <c r="B36" s="85"/>
+      <c r="A36" s="100" t="s">
+        <v>68</v>
+      </c>
+      <c r="B36" s="100"/>
       <c r="C36" s="27"/>
       <c r="D36" s="27"/>
       <c r="E36" s="27"/>
@@ -3980,7 +4181,7 @@
     </row>
     <row r="37" spans="1:20" ht="14.45" customHeight="1">
       <c r="A37" s="29" t="s">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="B37" s="44"/>
       <c r="C37" s="27"/>
@@ -4026,10 +4227,10 @@
     </row>
     <row r="39" spans="1:20" ht="15.6" customHeight="1">
       <c r="A39" s="46" t="s">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="B39" s="47" t="s">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="C39" s="48"/>
       <c r="D39" s="27"/>
@@ -4052,10 +4253,10 @@
     </row>
     <row r="40" spans="1:20" ht="29.1" customHeight="1">
       <c r="A40" s="46" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
       <c r="B40" s="47" t="s">
-        <v>48</v>
+        <v>72</v>
       </c>
       <c r="C40" s="48"/>
       <c r="D40" s="27"/>
@@ -4078,10 +4279,10 @@
     </row>
     <row r="41" spans="1:20" ht="15.6" customHeight="1">
       <c r="A41" s="46" t="s">
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="B41" s="47" t="s">
-        <v>50</v>
+        <v>74</v>
       </c>
       <c r="C41" s="49"/>
       <c r="D41" s="27"/>
@@ -4104,10 +4305,10 @@
     </row>
     <row r="42" spans="1:20" ht="15.6" customHeight="1">
       <c r="A42" s="46" t="s">
-        <v>51</v>
+        <v>75</v>
       </c>
       <c r="B42" s="47" t="s">
-        <v>52</v>
+        <v>76</v>
       </c>
       <c r="C42" s="50"/>
       <c r="D42" s="27"/>
@@ -4130,10 +4331,10 @@
     </row>
     <row r="43" spans="1:20" ht="15.6" customHeight="1">
       <c r="A43" s="46" t="s">
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="B43" s="47" t="s">
-        <v>54</v>
+        <v>78</v>
       </c>
       <c r="C43" s="51"/>
       <c r="D43" s="27"/>
@@ -4156,10 +4357,10 @@
     </row>
     <row r="44" spans="1:20" ht="14.45" customHeight="1">
       <c r="A44" s="46" t="s">
-        <v>55</v>
+        <v>79</v>
       </c>
       <c r="B44" s="47" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="C44" s="27"/>
       <c r="D44" s="27"/>
@@ -4182,10 +4383,10 @@
     </row>
     <row r="45" spans="1:20" ht="14.45" customHeight="1">
       <c r="A45" s="46" t="s">
-        <v>57</v>
+        <v>81</v>
       </c>
       <c r="B45" s="47" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="C45" s="27"/>
       <c r="D45" s="27"/>
@@ -4208,10 +4409,10 @@
     </row>
     <row r="46" spans="1:20" ht="14.45" customHeight="1">
       <c r="A46" s="46" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="B46" s="47" t="s">
-        <v>60</v>
+        <v>84</v>
       </c>
       <c r="C46" s="27"/>
       <c r="D46" s="27"/>
@@ -4234,10 +4435,10 @@
     </row>
     <row r="47" spans="1:20" ht="14.45" customHeight="1">
       <c r="A47" s="46" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="B47" s="47" t="s">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="C47" s="27"/>
       <c r="D47" s="27"/>
@@ -4260,10 +4461,10 @@
     </row>
     <row r="48" spans="1:20" ht="14.45" customHeight="1">
       <c r="A48" s="46" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="B48" s="47" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="C48" s="27"/>
       <c r="D48" s="27"/>
@@ -4286,10 +4487,10 @@
     </row>
     <row r="49" spans="1:20" ht="29.1" customHeight="1">
       <c r="A49" s="46" t="s">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="B49" s="52" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="C49" s="27"/>
       <c r="D49" s="27"/>
@@ -4312,10 +4513,10 @@
     </row>
     <row r="50" spans="1:20" ht="29.1" customHeight="1">
       <c r="A50" s="46" t="s">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="B50" s="52" t="s">
-        <v>68</v>
+        <v>92</v>
       </c>
       <c r="C50" s="27"/>
       <c r="D50" s="27"/>
@@ -4338,10 +4539,10 @@
     </row>
     <row r="51" spans="1:20" ht="14.45" customHeight="1">
       <c r="A51" s="46" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="B51" s="52" t="s">
-        <v>70</v>
+        <v>94</v>
       </c>
       <c r="C51" s="27"/>
       <c r="D51" s="27"/>
@@ -4364,10 +4565,10 @@
     </row>
     <row r="52" spans="1:20" ht="14.45" customHeight="1">
       <c r="A52" s="46" t="s">
-        <v>71</v>
+        <v>95</v>
       </c>
       <c r="B52" s="52" t="s">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="C52" s="27"/>
       <c r="D52" s="27"/>
@@ -4390,10 +4591,10 @@
     </row>
     <row r="53" spans="1:20" ht="14.45" customHeight="1">
       <c r="A53" s="46" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="B53" s="52" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="C53" s="27"/>
       <c r="D53" s="27"/>
@@ -4416,10 +4617,10 @@
     </row>
     <row r="54" spans="1:20" ht="14.45" customHeight="1">
       <c r="A54" s="46" t="s">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="B54" s="52" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="C54" s="27"/>
       <c r="D54" s="27"/>
@@ -4442,10 +4643,10 @@
     </row>
     <row r="55" spans="1:20" ht="14.45" customHeight="1">
       <c r="A55" s="46" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="B55" s="52" t="s">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="C55" s="27"/>
       <c r="D55" s="27"/>
@@ -4468,10 +4669,10 @@
     </row>
     <row r="56" spans="1:20" ht="29.1" customHeight="1">
       <c r="A56" s="53" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
       <c r="B56" s="52" t="s">
-        <v>80</v>
+        <v>104</v>
       </c>
       <c r="C56" s="27"/>
       <c r="D56" s="27"/>
@@ -4494,10 +4695,10 @@
     </row>
     <row r="57" spans="1:20" ht="14.45" customHeight="1">
       <c r="A57" s="53" t="s">
-        <v>81</v>
+        <v>105</v>
       </c>
       <c r="B57" s="52" t="s">
-        <v>82</v>
+        <v>106</v>
       </c>
       <c r="C57" s="27"/>
       <c r="D57" s="27"/>
@@ -4520,10 +4721,10 @@
     </row>
     <row r="58" spans="1:20" ht="29.1" customHeight="1">
       <c r="A58" s="46" t="s">
-        <v>83</v>
+        <v>107</v>
       </c>
       <c r="B58" s="52" t="s">
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="C58" s="27"/>
       <c r="D58" s="27"/>
@@ -4546,10 +4747,10 @@
     </row>
     <row r="59" spans="1:20" ht="14.45" customHeight="1">
       <c r="A59" s="53" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="B59" s="52" t="s">
-        <v>86</v>
+        <v>110</v>
       </c>
       <c r="C59" s="27"/>
       <c r="D59" s="27"/>
@@ -4572,10 +4773,10 @@
     </row>
     <row r="60" spans="1:20" ht="14.45" customHeight="1">
       <c r="A60" s="53" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="B60" s="52" t="s">
-        <v>88</v>
+        <v>112</v>
       </c>
       <c r="C60" s="27"/>
       <c r="D60" s="27"/>
@@ -4598,10 +4799,10 @@
     </row>
     <row r="61" spans="1:20" ht="14.45" customHeight="1">
       <c r="A61" s="53" t="s">
-        <v>89</v>
+        <v>113</v>
       </c>
       <c r="B61" s="52" t="s">
-        <v>90</v>
+        <v>114</v>
       </c>
       <c r="C61" s="27"/>
       <c r="D61" s="27"/>
@@ -4646,7 +4847,7 @@
     </row>
     <row r="63" spans="1:20" ht="18.600000000000001" customHeight="1">
       <c r="A63" s="54" t="s">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="B63" s="44"/>
       <c r="C63" s="27"/>
@@ -4692,10 +4893,10 @@
     </row>
     <row r="65" spans="1:20" ht="14.45" customHeight="1">
       <c r="A65" s="46" t="s">
-        <v>51</v>
+        <v>75</v>
       </c>
       <c r="B65" s="52" t="s">
-        <v>91</v>
+        <v>115</v>
       </c>
       <c r="C65" s="27"/>
       <c r="D65" s="27"/>
@@ -4718,10 +4919,10 @@
     </row>
     <row r="66" spans="1:20" ht="14.45" customHeight="1">
       <c r="A66" s="46" t="s">
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="B66" s="47" t="s">
-        <v>92</v>
+        <v>116</v>
       </c>
       <c r="C66" s="27"/>
       <c r="D66" s="27"/>
@@ -4744,10 +4945,10 @@
     </row>
     <row r="67" spans="1:20" ht="14.45" customHeight="1">
       <c r="A67" s="46" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="B67" s="44" t="s">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="C67" s="27"/>
       <c r="D67" s="27"/>
@@ -4770,10 +4971,10 @@
     </row>
     <row r="68" spans="1:20" ht="14.45" customHeight="1">
       <c r="A68" s="46" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="B68" s="47" t="s">
-        <v>94</v>
+        <v>118</v>
       </c>
       <c r="C68" s="27"/>
       <c r="D68" s="27"/>
@@ -4796,10 +4997,10 @@
     </row>
     <row r="69" spans="1:20" ht="14.45" customHeight="1">
       <c r="A69" s="46" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="B69" s="47" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="C69" s="27"/>
       <c r="D69" s="27"/>
@@ -4822,10 +5023,10 @@
     </row>
     <row r="70" spans="1:20" ht="14.45" customHeight="1">
       <c r="A70" s="46" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
       <c r="B70" s="44" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="C70" s="27"/>
       <c r="D70" s="27"/>
@@ -4848,10 +5049,10 @@
     </row>
     <row r="71" spans="1:20" ht="14.45" customHeight="1">
       <c r="A71" s="46" t="s">
-        <v>71</v>
+        <v>95</v>
       </c>
       <c r="B71" s="52" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="C71" s="27"/>
       <c r="D71" s="27"/>
@@ -4874,10 +5075,10 @@
     </row>
     <row r="72" spans="1:20" ht="14.45" customHeight="1">
       <c r="A72" s="46" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="B72" s="52" t="s">
-        <v>98</v>
+        <v>122</v>
       </c>
       <c r="C72" s="27"/>
       <c r="D72" s="27"/>
@@ -4900,10 +5101,10 @@
     </row>
     <row r="73" spans="1:20" ht="14.45" customHeight="1">
       <c r="A73" s="46" t="s">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="B73" s="52" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="C73" s="27"/>
       <c r="D73" s="27"/>
@@ -4926,10 +5127,10 @@
     </row>
     <row r="74" spans="1:20" ht="14.45" customHeight="1">
       <c r="A74" s="46" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="B74" s="52" t="s">
-        <v>100</v>
+        <v>124</v>
       </c>
       <c r="C74" s="27"/>
       <c r="D74" s="27"/>
@@ -4952,10 +5153,10 @@
     </row>
     <row r="75" spans="1:20" ht="14.45" customHeight="1">
       <c r="A75" s="53" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
       <c r="B75" s="52" t="s">
-        <v>101</v>
+        <v>125</v>
       </c>
       <c r="C75" s="27"/>
       <c r="D75" s="27"/>
@@ -4978,7 +5179,7 @@
     </row>
     <row r="76" spans="1:20" ht="14.45" customHeight="1">
       <c r="A76" s="53" t="s">
-        <v>81</v>
+        <v>105</v>
       </c>
       <c r="B76" s="52">
         <v>10</v>
@@ -5004,10 +5205,10 @@
     </row>
     <row r="77" spans="1:20" ht="87" customHeight="1">
       <c r="A77" s="46" t="s">
-        <v>83</v>
+        <v>107</v>
       </c>
       <c r="B77" s="52" t="s">
-        <v>102</v>
+        <v>126</v>
       </c>
       <c r="C77" s="27"/>
       <c r="D77" s="27"/>
@@ -5030,10 +5231,10 @@
     </row>
     <row r="78" spans="1:20" ht="29.1" customHeight="1">
       <c r="A78" s="53" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="B78" s="52" t="s">
-        <v>103</v>
+        <v>127</v>
       </c>
       <c r="C78" s="27"/>
       <c r="D78" s="27"/>
@@ -5056,10 +5257,10 @@
     </row>
     <row r="79" spans="1:20" ht="14.45" customHeight="1">
       <c r="A79" s="53" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="B79" s="52" t="s">
-        <v>104</v>
+        <v>128</v>
       </c>
       <c r="C79" s="27"/>
       <c r="D79" s="27"/>
@@ -5170,10 +5371,10 @@
     </row>
     <row r="84" spans="1:20" ht="14.45" customHeight="1">
       <c r="A84" s="46" t="s">
-        <v>105</v>
+        <v>129</v>
       </c>
       <c r="B84" s="47" t="s">
-        <v>106</v>
+        <v>130</v>
       </c>
       <c r="C84" s="27"/>
       <c r="D84" s="27"/>
@@ -5196,10 +5397,10 @@
     </row>
     <row r="85" spans="1:20" ht="29.1" customHeight="1">
       <c r="A85" s="46" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="B85" s="47" t="s">
-        <v>107</v>
+        <v>131</v>
       </c>
       <c r="C85" s="27"/>
       <c r="D85" s="27"/>
@@ -5222,10 +5423,10 @@
     </row>
     <row r="86" spans="1:20" ht="14.45" customHeight="1">
       <c r="A86" s="46" t="s">
-        <v>108</v>
+        <v>132</v>
       </c>
       <c r="B86" s="52" t="s">
-        <v>109</v>
+        <v>133</v>
       </c>
       <c r="C86" s="27"/>
       <c r="D86" s="27"/>
@@ -5248,10 +5449,10 @@
     </row>
     <row r="87" spans="1:20" ht="14.45" customHeight="1">
       <c r="A87" s="46" t="s">
-        <v>71</v>
+        <v>95</v>
       </c>
       <c r="B87" s="52" t="s">
-        <v>110</v>
+        <v>134</v>
       </c>
       <c r="C87" s="27"/>
       <c r="D87" s="27"/>
@@ -5274,10 +5475,10 @@
     </row>
     <row r="88" spans="1:20" ht="29.1" customHeight="1">
       <c r="A88" s="46" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="B88" s="52" t="s">
-        <v>111</v>
+        <v>135</v>
       </c>
       <c r="C88" s="27"/>
       <c r="D88" s="27"/>
@@ -5300,10 +5501,10 @@
     </row>
     <row r="89" spans="1:20" ht="14.45" customHeight="1">
       <c r="A89" s="46" t="s">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="B89" s="52" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="C89" s="27"/>
       <c r="D89" s="27"/>
@@ -5326,10 +5527,10 @@
     </row>
     <row r="90" spans="1:20" ht="14.45" customHeight="1">
       <c r="A90" s="46" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="B90" s="52" t="s">
-        <v>112</v>
+        <v>136</v>
       </c>
       <c r="C90" s="27"/>
       <c r="D90" s="27"/>
@@ -5352,10 +5553,10 @@
     </row>
     <row r="91" spans="1:20" ht="14.45" customHeight="1">
       <c r="A91" s="53" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
       <c r="B91" s="52" t="s">
-        <v>113</v>
+        <v>137</v>
       </c>
       <c r="C91" s="27"/>
       <c r="D91" s="27"/>
@@ -5378,7 +5579,7 @@
     </row>
     <row r="92" spans="1:20" ht="14.45" customHeight="1">
       <c r="A92" s="53" t="s">
-        <v>81</v>
+        <v>105</v>
       </c>
       <c r="B92" s="52">
         <v>2</v>
@@ -5404,10 +5605,10 @@
     </row>
     <row r="93" spans="1:20" ht="29.1" customHeight="1">
       <c r="A93" s="46" t="s">
-        <v>83</v>
+        <v>107</v>
       </c>
       <c r="B93" s="52" t="s">
-        <v>114</v>
+        <v>138</v>
       </c>
       <c r="C93" s="27"/>
       <c r="D93" s="27"/>
@@ -5430,10 +5631,10 @@
     </row>
     <row r="94" spans="1:20" ht="14.45" customHeight="1">
       <c r="A94" s="53" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="B94" s="52" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="C94" s="27"/>
       <c r="D94" s="27"/>
@@ -5456,10 +5657,10 @@
     </row>
     <row r="95" spans="1:20" ht="14.45" customHeight="1">
       <c r="A95" s="53" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="B95" s="52" t="s">
-        <v>104</v>
+        <v>128</v>
       </c>
       <c r="C95" s="27"/>
       <c r="D95" s="27"/>
@@ -5811,10 +6012,10 @@
       <c r="T110" s="27"/>
     </row>
     <row r="111" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A111" s="86" t="s">
-        <v>116</v>
-      </c>
-      <c r="B111" s="86"/>
+      <c r="A111" s="88" t="s">
+        <v>140</v>
+      </c>
+      <c r="B111" s="88"/>
       <c r="C111" s="27"/>
       <c r="D111" s="27"/>
       <c r="E111" s="27"/>
@@ -5836,7 +6037,7 @@
     </row>
     <row r="112" spans="1:20" ht="14.45" customHeight="1">
       <c r="A112" s="29" t="s">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="B112" s="27"/>
       <c r="C112" s="27"/>
@@ -5882,13 +6083,13 @@
     </row>
     <row r="114" spans="1:20" ht="15.6" customHeight="1">
       <c r="A114" s="56" t="s">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="B114" s="57" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="C114" s="56" t="s">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="D114" s="27"/>
       <c r="E114" s="27"/>
@@ -5910,13 +6111,13 @@
     </row>
     <row r="115" spans="1:20" ht="15.6" customHeight="1">
       <c r="A115" s="58" t="s">
-        <v>119</v>
+        <v>143</v>
       </c>
       <c r="B115" s="59" t="s">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="C115" s="60" t="s">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="D115" s="27"/>
       <c r="E115" s="27"/>
@@ -5938,13 +6139,13 @@
     </row>
     <row r="116" spans="1:20" ht="15.6" customHeight="1">
       <c r="A116" s="58" t="s">
-        <v>122</v>
+        <v>146</v>
       </c>
       <c r="B116" s="59" t="s">
-        <v>123</v>
+        <v>147</v>
       </c>
       <c r="C116" s="60" t="s">
-        <v>124</v>
+        <v>148</v>
       </c>
       <c r="D116" s="27"/>
       <c r="E116" s="27"/>
@@ -5966,13 +6167,13 @@
     </row>
     <row r="117" spans="1:20" ht="15.6" customHeight="1">
       <c r="A117" s="58" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="B117" s="59" t="s">
-        <v>125</v>
+        <v>149</v>
       </c>
       <c r="C117" s="60" t="s">
-        <v>126</v>
+        <v>150</v>
       </c>
       <c r="D117" s="27"/>
       <c r="E117" s="27"/>
@@ -5994,13 +6195,13 @@
     </row>
     <row r="118" spans="1:20" ht="15.6" customHeight="1">
       <c r="A118" s="58" t="s">
-        <v>127</v>
+        <v>151</v>
       </c>
       <c r="B118" s="59" t="s">
-        <v>128</v>
+        <v>152</v>
       </c>
       <c r="C118" s="60" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
       <c r="D118" s="27"/>
       <c r="E118" s="27"/>
@@ -6022,13 +6223,13 @@
     </row>
     <row r="119" spans="1:20" ht="15.6" customHeight="1">
       <c r="A119" s="58" t="s">
-        <v>130</v>
+        <v>154</v>
       </c>
       <c r="B119" s="61" t="s">
-        <v>131</v>
+        <v>155</v>
       </c>
       <c r="C119" s="62" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="D119" s="27"/>
       <c r="E119" s="27"/>
@@ -6050,13 +6251,13 @@
     </row>
     <row r="120" spans="1:20" ht="15.6" customHeight="1">
       <c r="A120" s="58" t="s">
-        <v>133</v>
+        <v>157</v>
       </c>
       <c r="B120" s="59" t="s">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="C120" s="60" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="D120" s="27"/>
       <c r="E120" s="27"/>
@@ -6078,13 +6279,13 @@
     </row>
     <row r="121" spans="1:20" ht="15.6" customHeight="1">
       <c r="A121" s="58" t="s">
-        <v>136</v>
+        <v>160</v>
       </c>
       <c r="B121" s="61" t="s">
-        <v>137</v>
+        <v>161</v>
       </c>
       <c r="C121" s="60" t="s">
-        <v>138</v>
+        <v>162</v>
       </c>
       <c r="D121" s="27"/>
       <c r="E121" s="27"/>
@@ -6106,13 +6307,13 @@
     </row>
     <row r="122" spans="1:20" ht="15.6" customHeight="1">
       <c r="A122" s="58" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
       <c r="B122" s="59" t="s">
-        <v>140</v>
+        <v>164</v>
       </c>
       <c r="C122" s="60" t="s">
-        <v>141</v>
+        <v>165</v>
       </c>
       <c r="D122" s="27"/>
       <c r="E122" s="27"/>
@@ -6134,13 +6335,13 @@
     </row>
     <row r="123" spans="1:20" ht="15.6" customHeight="1">
       <c r="A123" s="58" t="s">
-        <v>142</v>
+        <v>166</v>
       </c>
       <c r="B123" s="59" t="s">
-        <v>143</v>
+        <v>167</v>
       </c>
       <c r="C123" s="60" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="D123" s="27"/>
       <c r="E123" s="27"/>
@@ -6162,13 +6363,13 @@
     </row>
     <row r="124" spans="1:20" ht="15.6" customHeight="1">
       <c r="A124" s="58" t="s">
-        <v>145</v>
+        <v>169</v>
       </c>
       <c r="B124" s="59" t="s">
-        <v>146</v>
+        <v>170</v>
       </c>
       <c r="C124" s="60" t="s">
-        <v>147</v>
+        <v>171</v>
       </c>
       <c r="D124" s="27"/>
       <c r="E124" s="27"/>
@@ -6190,13 +6391,13 @@
     </row>
     <row r="125" spans="1:20" ht="15.6" customHeight="1">
       <c r="A125" s="58" t="s">
-        <v>148</v>
+        <v>172</v>
       </c>
       <c r="B125" s="61" t="s">
-        <v>149</v>
+        <v>173</v>
       </c>
       <c r="C125" s="60" t="s">
-        <v>150</v>
+        <v>174</v>
       </c>
       <c r="D125" s="27"/>
       <c r="E125" s="27"/>
@@ -6218,13 +6419,13 @@
     </row>
     <row r="126" spans="1:20" ht="15.6" customHeight="1">
       <c r="A126" s="58" t="s">
-        <v>151</v>
+        <v>175</v>
       </c>
       <c r="B126" s="28" t="s">
-        <v>152</v>
+        <v>176</v>
       </c>
       <c r="C126" s="60" t="s">
-        <v>153</v>
+        <v>177</v>
       </c>
       <c r="D126" s="27"/>
       <c r="E126" s="27"/>
@@ -6246,13 +6447,13 @@
     </row>
     <row r="127" spans="1:20" ht="30.95" customHeight="1">
       <c r="A127" s="58" t="s">
-        <v>154</v>
+        <v>178</v>
       </c>
       <c r="B127" s="59" t="s">
-        <v>155</v>
+        <v>179</v>
       </c>
       <c r="C127" s="60" t="s">
-        <v>156</v>
+        <v>180</v>
       </c>
       <c r="D127" s="27"/>
       <c r="E127" s="27"/>
@@ -6274,13 +6475,13 @@
     </row>
     <row r="128" spans="1:20" ht="15.6" customHeight="1">
       <c r="A128" s="58" t="s">
-        <v>157</v>
+        <v>181</v>
       </c>
       <c r="B128" s="63" t="s">
-        <v>158</v>
+        <v>182</v>
       </c>
       <c r="C128" s="60" t="s">
-        <v>159</v>
+        <v>183</v>
       </c>
       <c r="D128" s="27"/>
       <c r="E128" s="27"/>
@@ -6302,13 +6503,13 @@
     </row>
     <row r="129" spans="1:20" ht="15.6" customHeight="1">
       <c r="A129" s="58" t="s">
-        <v>160</v>
+        <v>184</v>
       </c>
       <c r="B129" s="59" t="s">
-        <v>161</v>
+        <v>185</v>
       </c>
       <c r="C129" s="60" t="s">
-        <v>162</v>
+        <v>186</v>
       </c>
       <c r="D129" s="27"/>
       <c r="E129" s="27"/>
@@ -6330,13 +6531,13 @@
     </row>
     <row r="130" spans="1:20" ht="15.6" customHeight="1">
       <c r="A130" s="58" t="s">
-        <v>163</v>
+        <v>187</v>
       </c>
       <c r="B130" s="61" t="s">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="C130" s="60" t="s">
-        <v>165</v>
+        <v>189</v>
       </c>
       <c r="D130" s="27"/>
       <c r="E130" s="27"/>
@@ -6358,13 +6559,13 @@
     </row>
     <row r="131" spans="1:20" ht="15.6" customHeight="1">
       <c r="A131" s="58" t="s">
-        <v>166</v>
+        <v>190</v>
       </c>
       <c r="B131" s="61" t="s">
-        <v>167</v>
+        <v>191</v>
       </c>
       <c r="C131" s="60" t="s">
-        <v>168</v>
+        <v>192</v>
       </c>
       <c r="D131" s="27"/>
       <c r="E131" s="27"/>
@@ -6386,13 +6587,13 @@
     </row>
     <row r="132" spans="1:20" ht="15.6" customHeight="1">
       <c r="A132" s="58" t="s">
-        <v>169</v>
+        <v>193</v>
       </c>
       <c r="B132" s="59" t="s">
-        <v>170</v>
+        <v>194</v>
       </c>
       <c r="C132" s="60" t="s">
-        <v>171</v>
+        <v>195</v>
       </c>
       <c r="D132" s="27"/>
       <c r="E132" s="27"/>
@@ -6414,13 +6615,13 @@
     </row>
     <row r="133" spans="1:20" ht="15.6" customHeight="1">
       <c r="A133" s="58" t="s">
-        <v>172</v>
+        <v>196</v>
       </c>
       <c r="B133" s="59" t="s">
-        <v>173</v>
+        <v>197</v>
       </c>
       <c r="C133" s="60" t="s">
-        <v>174</v>
+        <v>198</v>
       </c>
       <c r="D133" s="27"/>
       <c r="E133" s="27"/>
@@ -6552,7 +6753,7 @@
     </row>
     <row r="139" spans="1:20" ht="14.45" customHeight="1">
       <c r="A139" s="27" t="s">
-        <v>175</v>
+        <v>199</v>
       </c>
       <c r="B139" s="27"/>
       <c r="C139" s="27"/>
@@ -6620,111 +6821,111 @@
     </row>
     <row r="142" spans="1:20" s="22" customFormat="1" ht="15.95" customHeight="1">
       <c r="A142" s="64" t="s">
-        <v>176</v>
+        <v>200</v>
       </c>
       <c r="B142" s="64" t="s">
-        <v>177</v>
+        <v>201</v>
       </c>
       <c r="C142" s="64" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="D142" s="64" t="s">
-        <v>179</v>
+        <v>203</v>
       </c>
       <c r="E142" s="64" t="s">
-        <v>180</v>
+        <v>204</v>
       </c>
       <c r="F142" s="64" t="s">
-        <v>181</v>
+        <v>205</v>
       </c>
       <c r="G142" s="64" t="s">
-        <v>182</v>
+        <v>206</v>
       </c>
       <c r="H142" s="64" t="s">
-        <v>183</v>
+        <v>207</v>
       </c>
       <c r="I142" s="64" t="s">
-        <v>184</v>
+        <v>208</v>
       </c>
       <c r="J142" s="64" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="K142" s="64" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="L142" s="64" t="s">
-        <v>186</v>
+        <v>210</v>
       </c>
       <c r="M142" s="64" t="s">
-        <v>187</v>
+        <v>211</v>
       </c>
       <c r="N142" s="64" t="s">
-        <v>188</v>
+        <v>212</v>
       </c>
       <c r="O142" s="64" t="s">
-        <v>189</v>
+        <v>213</v>
       </c>
       <c r="P142" s="64" t="s">
-        <v>190</v>
+        <v>214</v>
       </c>
       <c r="Q142" s="64" t="s">
-        <v>191</v>
+        <v>215</v>
       </c>
       <c r="R142" s="64" t="s">
-        <v>192</v>
+        <v>216</v>
       </c>
       <c r="S142" s="64" t="s">
-        <v>193</v>
+        <v>217</v>
       </c>
       <c r="T142" s="64"/>
     </row>
     <row r="143" spans="1:20" ht="14.45" customHeight="1">
       <c r="A143" s="27" t="s">
-        <v>194</v>
+        <v>218</v>
       </c>
       <c r="B143" s="27" t="s">
-        <v>195</v>
+        <v>219</v>
       </c>
       <c r="C143" s="27" t="s">
-        <v>196</v>
+        <v>220</v>
       </c>
       <c r="D143" s="27" t="s">
-        <v>197</v>
+        <v>221</v>
       </c>
       <c r="E143" s="27" t="s">
-        <v>198</v>
+        <v>222</v>
       </c>
       <c r="F143" s="27" t="s">
-        <v>199</v>
+        <v>223</v>
       </c>
       <c r="G143" s="27" t="s">
-        <v>200</v>
+        <v>224</v>
       </c>
       <c r="H143" s="27" t="s">
-        <v>201</v>
+        <v>225</v>
       </c>
       <c r="I143" s="27" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="J143" s="27" t="s">
-        <v>203</v>
+        <v>227</v>
       </c>
       <c r="K143" s="27" t="s">
-        <v>204</v>
+        <v>228</v>
       </c>
       <c r="L143" s="27"/>
       <c r="M143" s="27" t="s">
-        <v>205</v>
+        <v>229</v>
       </c>
       <c r="N143" s="27"/>
       <c r="O143" s="27" t="s">
-        <v>206</v>
+        <v>230</v>
       </c>
       <c r="P143" s="27"/>
       <c r="Q143" s="27"/>
       <c r="R143" s="27"/>
       <c r="S143" s="27" t="s">
-        <v>207</v>
+        <v>231</v>
       </c>
       <c r="T143" s="27"/>
     </row>
@@ -6735,33 +6936,33 @@
       <c r="D144" s="27"/>
       <c r="E144" s="27"/>
       <c r="F144" s="27" t="s">
-        <v>199</v>
+        <v>223</v>
       </c>
       <c r="G144" s="27" t="s">
-        <v>200</v>
+        <v>224</v>
       </c>
       <c r="H144" s="27" t="s">
-        <v>201</v>
+        <v>225</v>
       </c>
       <c r="I144" s="27" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="J144" s="27" t="s">
-        <v>208</v>
+        <v>232</v>
       </c>
       <c r="K144" s="27" t="s">
-        <v>209</v>
+        <v>233</v>
       </c>
       <c r="L144" s="27" t="s">
-        <v>210</v>
+        <v>234</v>
       </c>
       <c r="M144" s="27" t="s">
-        <v>205</v>
+        <v>229</v>
       </c>
       <c r="N144" s="27"/>
       <c r="O144" s="27"/>
       <c r="P144" s="27" t="s">
-        <v>210</v>
+        <v>234</v>
       </c>
       <c r="Q144" s="27"/>
       <c r="R144" s="27"/>
@@ -6775,37 +6976,37 @@
       <c r="D145" s="27"/>
       <c r="E145" s="27"/>
       <c r="F145" s="27" t="s">
-        <v>199</v>
+        <v>223</v>
       </c>
       <c r="G145" s="27" t="s">
-        <v>200</v>
+        <v>224</v>
       </c>
       <c r="H145" s="27" t="s">
-        <v>201</v>
+        <v>225</v>
       </c>
       <c r="I145" s="27" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="J145" s="27" t="s">
-        <v>211</v>
+        <v>235</v>
       </c>
       <c r="K145" s="27" t="s">
-        <v>204</v>
+        <v>228</v>
       </c>
       <c r="L145" s="27"/>
       <c r="M145" s="27" t="s">
-        <v>205</v>
+        <v>229</v>
       </c>
       <c r="N145" s="27"/>
       <c r="O145" s="27" t="s">
-        <v>212</v>
+        <v>236</v>
       </c>
       <c r="P145" s="27"/>
       <c r="Q145" s="27" t="s">
-        <v>213</v>
+        <v>237</v>
       </c>
       <c r="R145" s="27" t="s">
-        <v>214</v>
+        <v>238</v>
       </c>
       <c r="S145" s="27"/>
       <c r="T145" s="27"/>
@@ -7099,7 +7300,7 @@
     <row r="159" spans="1:20" ht="15.6" customHeight="1">
       <c r="A159" s="27"/>
       <c r="B159" s="55" t="s">
-        <v>215</v>
+        <v>239</v>
       </c>
       <c r="C159" s="27"/>
       <c r="D159" s="27"/>
@@ -7144,16 +7345,16 @@
     </row>
     <row r="161" spans="1:20" ht="14.45" customHeight="1">
       <c r="A161" s="65" t="s">
-        <v>216</v>
+        <v>240</v>
       </c>
       <c r="B161" s="65" t="s">
-        <v>217</v>
+        <v>241</v>
       </c>
       <c r="C161" s="65" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="D161" s="65" t="s">
-        <v>218</v>
+        <v>242</v>
       </c>
       <c r="E161" s="27"/>
       <c r="F161" s="27"/>
@@ -7173,17 +7374,17 @@
       <c r="T161" s="27"/>
     </row>
     <row r="162" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A162" s="90" t="s">
-        <v>219</v>
-      </c>
-      <c r="B162" s="79" t="e" vm="1">
+      <c r="A162" s="89" t="s">
+        <v>243</v>
+      </c>
+      <c r="B162" s="82" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
       <c r="C162" s="76" t="s">
-        <v>220</v>
+        <v>244</v>
       </c>
       <c r="D162" s="76" t="s">
-        <v>221</v>
+        <v>245</v>
       </c>
       <c r="E162" s="27"/>
       <c r="F162" s="27"/>
@@ -7203,8 +7404,8 @@
       <c r="T162" s="27"/>
     </row>
     <row r="163" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A163" s="91"/>
-      <c r="B163" s="80"/>
+      <c r="A163" s="90"/>
+      <c r="B163" s="83"/>
       <c r="C163" s="77"/>
       <c r="D163" s="77"/>
       <c r="E163" s="27"/>
@@ -7225,8 +7426,8 @@
       <c r="T163" s="27"/>
     </row>
     <row r="164" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A164" s="91"/>
-      <c r="B164" s="80"/>
+      <c r="A164" s="90"/>
+      <c r="B164" s="83"/>
       <c r="C164" s="77"/>
       <c r="D164" s="77"/>
       <c r="E164" s="27"/>
@@ -7247,8 +7448,8 @@
       <c r="T164" s="27"/>
     </row>
     <row r="165" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A165" s="91"/>
-      <c r="B165" s="80"/>
+      <c r="A165" s="90"/>
+      <c r="B165" s="83"/>
       <c r="C165" s="77"/>
       <c r="D165" s="77"/>
       <c r="E165" s="27"/>
@@ -7269,8 +7470,8 @@
       <c r="T165" s="27"/>
     </row>
     <row r="166" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A166" s="91"/>
-      <c r="B166" s="80"/>
+      <c r="A166" s="90"/>
+      <c r="B166" s="83"/>
       <c r="C166" s="77"/>
       <c r="D166" s="77"/>
       <c r="E166" s="27"/>
@@ -7291,8 +7492,8 @@
       <c r="T166" s="27"/>
     </row>
     <row r="167" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A167" s="91"/>
-      <c r="B167" s="80"/>
+      <c r="A167" s="90"/>
+      <c r="B167" s="83"/>
       <c r="C167" s="77"/>
       <c r="D167" s="77"/>
       <c r="E167" s="27"/>
@@ -7313,8 +7514,8 @@
       <c r="T167" s="27"/>
     </row>
     <row r="168" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A168" s="91"/>
-      <c r="B168" s="80"/>
+      <c r="A168" s="90"/>
+      <c r="B168" s="83"/>
       <c r="C168" s="77"/>
       <c r="D168" s="77"/>
       <c r="E168" s="27"/>
@@ -7335,8 +7536,8 @@
       <c r="T168" s="27"/>
     </row>
     <row r="169" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A169" s="91"/>
-      <c r="B169" s="80"/>
+      <c r="A169" s="90"/>
+      <c r="B169" s="83"/>
       <c r="C169" s="77"/>
       <c r="D169" s="77"/>
       <c r="E169" s="27"/>
@@ -7357,8 +7558,8 @@
       <c r="T169" s="27"/>
     </row>
     <row r="170" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A170" s="91"/>
-      <c r="B170" s="80"/>
+      <c r="A170" s="90"/>
+      <c r="B170" s="83"/>
       <c r="C170" s="77"/>
       <c r="D170" s="77"/>
       <c r="E170" s="27"/>
@@ -7379,8 +7580,8 @@
       <c r="T170" s="27"/>
     </row>
     <row r="171" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A171" s="91"/>
-      <c r="B171" s="80"/>
+      <c r="A171" s="90"/>
+      <c r="B171" s="83"/>
       <c r="C171" s="77"/>
       <c r="D171" s="77"/>
       <c r="E171" s="27"/>
@@ -7401,8 +7602,8 @@
       <c r="T171" s="27"/>
     </row>
     <row r="172" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A172" s="91"/>
-      <c r="B172" s="80"/>
+      <c r="A172" s="90"/>
+      <c r="B172" s="83"/>
       <c r="C172" s="77"/>
       <c r="D172" s="77"/>
       <c r="E172" s="27"/>
@@ -7423,8 +7624,8 @@
       <c r="T172" s="27"/>
     </row>
     <row r="173" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A173" s="91"/>
-      <c r="B173" s="80"/>
+      <c r="A173" s="90"/>
+      <c r="B173" s="83"/>
       <c r="C173" s="77"/>
       <c r="D173" s="77"/>
       <c r="E173" s="27"/>
@@ -7445,8 +7646,8 @@
       <c r="T173" s="27"/>
     </row>
     <row r="174" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A174" s="91"/>
-      <c r="B174" s="80"/>
+      <c r="A174" s="90"/>
+      <c r="B174" s="83"/>
       <c r="C174" s="77"/>
       <c r="D174" s="77"/>
       <c r="E174" s="27"/>
@@ -7467,8 +7668,8 @@
       <c r="T174" s="27"/>
     </row>
     <row r="175" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A175" s="92"/>
-      <c r="B175" s="81"/>
+      <c r="A175" s="91"/>
+      <c r="B175" s="84"/>
       <c r="C175" s="78"/>
       <c r="D175" s="78"/>
       <c r="E175" s="27"/>
@@ -7489,17 +7690,17 @@
       <c r="T175" s="27"/>
     </row>
     <row r="176" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A176" s="90" t="s">
-        <v>222</v>
-      </c>
-      <c r="B176" s="79" t="e" vm="2">
+      <c r="A176" s="89" t="s">
+        <v>246</v>
+      </c>
+      <c r="B176" s="82" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
       <c r="C176" s="76" t="s">
-        <v>223</v>
+        <v>247</v>
       </c>
       <c r="D176" s="76" t="s">
-        <v>224</v>
+        <v>248</v>
       </c>
       <c r="E176" s="27"/>
       <c r="F176" s="27"/>
@@ -7519,8 +7720,8 @@
       <c r="T176" s="27"/>
     </row>
     <row r="177" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A177" s="91"/>
-      <c r="B177" s="80"/>
+      <c r="A177" s="90"/>
+      <c r="B177" s="83"/>
       <c r="C177" s="77"/>
       <c r="D177" s="77"/>
       <c r="E177" s="27"/>
@@ -7541,8 +7742,8 @@
       <c r="T177" s="27"/>
     </row>
     <row r="178" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A178" s="91"/>
-      <c r="B178" s="80"/>
+      <c r="A178" s="90"/>
+      <c r="B178" s="83"/>
       <c r="C178" s="77"/>
       <c r="D178" s="77"/>
       <c r="E178" s="27"/>
@@ -7563,8 +7764,8 @@
       <c r="T178" s="27"/>
     </row>
     <row r="179" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A179" s="91"/>
-      <c r="B179" s="80"/>
+      <c r="A179" s="90"/>
+      <c r="B179" s="83"/>
       <c r="C179" s="77"/>
       <c r="D179" s="77"/>
       <c r="E179" s="27"/>
@@ -7585,8 +7786,8 @@
       <c r="T179" s="27"/>
     </row>
     <row r="180" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A180" s="91"/>
-      <c r="B180" s="80"/>
+      <c r="A180" s="90"/>
+      <c r="B180" s="83"/>
       <c r="C180" s="77"/>
       <c r="D180" s="77"/>
       <c r="E180" s="27"/>
@@ -7607,8 +7808,8 @@
       <c r="T180" s="27"/>
     </row>
     <row r="181" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A181" s="91"/>
-      <c r="B181" s="80"/>
+      <c r="A181" s="90"/>
+      <c r="B181" s="83"/>
       <c r="C181" s="77"/>
       <c r="D181" s="77"/>
       <c r="E181" s="27"/>
@@ -7629,8 +7830,8 @@
       <c r="T181" s="27"/>
     </row>
     <row r="182" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A182" s="91"/>
-      <c r="B182" s="80"/>
+      <c r="A182" s="90"/>
+      <c r="B182" s="83"/>
       <c r="C182" s="77"/>
       <c r="D182" s="77"/>
       <c r="E182" s="27"/>
@@ -7651,8 +7852,8 @@
       <c r="T182" s="27"/>
     </row>
     <row r="183" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A183" s="91"/>
-      <c r="B183" s="80"/>
+      <c r="A183" s="90"/>
+      <c r="B183" s="83"/>
       <c r="C183" s="77"/>
       <c r="D183" s="77"/>
       <c r="E183" s="27"/>
@@ -7673,8 +7874,8 @@
       <c r="T183" s="27"/>
     </row>
     <row r="184" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A184" s="91"/>
-      <c r="B184" s="80"/>
+      <c r="A184" s="90"/>
+      <c r="B184" s="83"/>
       <c r="C184" s="77"/>
       <c r="D184" s="77"/>
       <c r="E184" s="27"/>
@@ -7695,8 +7896,8 @@
       <c r="T184" s="27"/>
     </row>
     <row r="185" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A185" s="91"/>
-      <c r="B185" s="80"/>
+      <c r="A185" s="90"/>
+      <c r="B185" s="83"/>
       <c r="C185" s="77"/>
       <c r="D185" s="77"/>
       <c r="E185" s="27"/>
@@ -7717,8 +7918,8 @@
       <c r="T185" s="27"/>
     </row>
     <row r="186" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A186" s="91"/>
-      <c r="B186" s="80"/>
+      <c r="A186" s="90"/>
+      <c r="B186" s="83"/>
       <c r="C186" s="77"/>
       <c r="D186" s="77"/>
       <c r="E186" s="27"/>
@@ -7739,8 +7940,8 @@
       <c r="T186" s="27"/>
     </row>
     <row r="187" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A187" s="91"/>
-      <c r="B187" s="80"/>
+      <c r="A187" s="90"/>
+      <c r="B187" s="83"/>
       <c r="C187" s="77"/>
       <c r="D187" s="77"/>
       <c r="E187" s="27"/>
@@ -7761,8 +7962,8 @@
       <c r="T187" s="27"/>
     </row>
     <row r="188" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A188" s="91"/>
-      <c r="B188" s="80"/>
+      <c r="A188" s="90"/>
+      <c r="B188" s="83"/>
       <c r="C188" s="77"/>
       <c r="D188" s="77"/>
       <c r="E188" s="27"/>
@@ -7783,8 +7984,8 @@
       <c r="T188" s="27"/>
     </row>
     <row r="189" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A189" s="92"/>
-      <c r="B189" s="81"/>
+      <c r="A189" s="91"/>
+      <c r="B189" s="84"/>
       <c r="C189" s="78"/>
       <c r="D189" s="78"/>
       <c r="E189" s="27"/>
@@ -7805,17 +8006,17 @@
       <c r="T189" s="27"/>
     </row>
     <row r="190" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A190" s="90" t="s">
-        <v>225</v>
-      </c>
-      <c r="B190" s="79" t="e" vm="3">
+      <c r="A190" s="89" t="s">
+        <v>249</v>
+      </c>
+      <c r="B190" s="82" t="e" vm="3">
         <v>#VALUE!</v>
       </c>
       <c r="C190" s="76" t="s">
-        <v>226</v>
+        <v>250</v>
       </c>
       <c r="D190" s="76" t="s">
-        <v>227</v>
+        <v>251</v>
       </c>
       <c r="E190" s="27"/>
       <c r="F190" s="27"/>
@@ -7835,8 +8036,8 @@
       <c r="T190" s="27"/>
     </row>
     <row r="191" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A191" s="91"/>
-      <c r="B191" s="80"/>
+      <c r="A191" s="90"/>
+      <c r="B191" s="83"/>
       <c r="C191" s="77"/>
       <c r="D191" s="77"/>
       <c r="E191" s="27"/>
@@ -7857,8 +8058,8 @@
       <c r="T191" s="27"/>
     </row>
     <row r="192" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A192" s="91"/>
-      <c r="B192" s="80"/>
+      <c r="A192" s="90"/>
+      <c r="B192" s="83"/>
       <c r="C192" s="77"/>
       <c r="D192" s="77"/>
       <c r="E192" s="27"/>
@@ -7879,8 +8080,8 @@
       <c r="T192" s="27"/>
     </row>
     <row r="193" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A193" s="91"/>
-      <c r="B193" s="80"/>
+      <c r="A193" s="90"/>
+      <c r="B193" s="83"/>
       <c r="C193" s="77"/>
       <c r="D193" s="77"/>
       <c r="E193" s="27"/>
@@ -7901,8 +8102,8 @@
       <c r="T193" s="27"/>
     </row>
     <row r="194" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A194" s="91"/>
-      <c r="B194" s="80"/>
+      <c r="A194" s="90"/>
+      <c r="B194" s="83"/>
       <c r="C194" s="77"/>
       <c r="D194" s="77"/>
       <c r="E194" s="27"/>
@@ -7923,8 +8124,8 @@
       <c r="T194" s="27"/>
     </row>
     <row r="195" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A195" s="91"/>
-      <c r="B195" s="80"/>
+      <c r="A195" s="90"/>
+      <c r="B195" s="83"/>
       <c r="C195" s="77"/>
       <c r="D195" s="77"/>
       <c r="E195" s="27"/>
@@ -7945,8 +8146,8 @@
       <c r="T195" s="27"/>
     </row>
     <row r="196" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A196" s="91"/>
-      <c r="B196" s="80"/>
+      <c r="A196" s="90"/>
+      <c r="B196" s="83"/>
       <c r="C196" s="77"/>
       <c r="D196" s="77"/>
       <c r="E196" s="27"/>
@@ -7967,8 +8168,8 @@
       <c r="T196" s="27"/>
     </row>
     <row r="197" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A197" s="91"/>
-      <c r="B197" s="80"/>
+      <c r="A197" s="90"/>
+      <c r="B197" s="83"/>
       <c r="C197" s="77"/>
       <c r="D197" s="77"/>
       <c r="E197" s="27"/>
@@ -7989,8 +8190,8 @@
       <c r="T197" s="27"/>
     </row>
     <row r="198" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A198" s="91"/>
-      <c r="B198" s="80"/>
+      <c r="A198" s="90"/>
+      <c r="B198" s="83"/>
       <c r="C198" s="77"/>
       <c r="D198" s="77"/>
       <c r="E198" s="27"/>
@@ -8011,8 +8212,8 @@
       <c r="T198" s="27"/>
     </row>
     <row r="199" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A199" s="91"/>
-      <c r="B199" s="80"/>
+      <c r="A199" s="90"/>
+      <c r="B199" s="83"/>
       <c r="C199" s="77"/>
       <c r="D199" s="77"/>
       <c r="E199" s="27"/>
@@ -8033,8 +8234,8 @@
       <c r="T199" s="27"/>
     </row>
     <row r="200" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A200" s="91"/>
-      <c r="B200" s="80"/>
+      <c r="A200" s="90"/>
+      <c r="B200" s="83"/>
       <c r="C200" s="77"/>
       <c r="D200" s="77"/>
       <c r="E200" s="27"/>
@@ -8055,8 +8256,8 @@
       <c r="T200" s="27"/>
     </row>
     <row r="201" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A201" s="91"/>
-      <c r="B201" s="80"/>
+      <c r="A201" s="90"/>
+      <c r="B201" s="83"/>
       <c r="C201" s="77"/>
       <c r="D201" s="77"/>
       <c r="E201" s="27"/>
@@ -8077,8 +8278,8 @@
       <c r="T201" s="27"/>
     </row>
     <row r="202" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A202" s="91"/>
-      <c r="B202" s="80"/>
+      <c r="A202" s="90"/>
+      <c r="B202" s="83"/>
       <c r="C202" s="77"/>
       <c r="D202" s="77"/>
       <c r="E202" s="27"/>
@@ -8099,8 +8300,8 @@
       <c r="T202" s="27"/>
     </row>
     <row r="203" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A203" s="92"/>
-      <c r="B203" s="81"/>
+      <c r="A203" s="91"/>
+      <c r="B203" s="84"/>
       <c r="C203" s="78"/>
       <c r="D203" s="78"/>
       <c r="E203" s="27"/>
@@ -8121,17 +8322,17 @@
       <c r="T203" s="27"/>
     </row>
     <row r="204" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A204" s="90" t="s">
-        <v>228</v>
-      </c>
-      <c r="B204" s="79" t="e" vm="4">
+      <c r="A204" s="89" t="s">
+        <v>252</v>
+      </c>
+      <c r="B204" s="82" t="e" vm="4">
         <v>#VALUE!</v>
       </c>
       <c r="C204" s="76" t="s">
-        <v>229</v>
+        <v>253</v>
       </c>
       <c r="D204" s="76" t="s">
-        <v>230</v>
+        <v>254</v>
       </c>
       <c r="E204" s="27"/>
       <c r="F204" s="27"/>
@@ -8151,8 +8352,8 @@
       <c r="T204" s="27"/>
     </row>
     <row r="205" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A205" s="91"/>
-      <c r="B205" s="80"/>
+      <c r="A205" s="90"/>
+      <c r="B205" s="83"/>
       <c r="C205" s="77"/>
       <c r="D205" s="77"/>
       <c r="E205" s="27"/>
@@ -8173,8 +8374,8 @@
       <c r="T205" s="27"/>
     </row>
     <row r="206" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A206" s="91"/>
-      <c r="B206" s="80"/>
+      <c r="A206" s="90"/>
+      <c r="B206" s="83"/>
       <c r="C206" s="77"/>
       <c r="D206" s="77"/>
       <c r="E206" s="27"/>
@@ -8195,8 +8396,8 @@
       <c r="T206" s="27"/>
     </row>
     <row r="207" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A207" s="91"/>
-      <c r="B207" s="80"/>
+      <c r="A207" s="90"/>
+      <c r="B207" s="83"/>
       <c r="C207" s="77"/>
       <c r="D207" s="77"/>
       <c r="E207" s="27"/>
@@ -8217,8 +8418,8 @@
       <c r="T207" s="27"/>
     </row>
     <row r="208" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A208" s="91"/>
-      <c r="B208" s="80"/>
+      <c r="A208" s="90"/>
+      <c r="B208" s="83"/>
       <c r="C208" s="77"/>
       <c r="D208" s="77"/>
       <c r="E208" s="27"/>
@@ -8239,8 +8440,8 @@
       <c r="T208" s="27"/>
     </row>
     <row r="209" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A209" s="91"/>
-      <c r="B209" s="80"/>
+      <c r="A209" s="90"/>
+      <c r="B209" s="83"/>
       <c r="C209" s="77"/>
       <c r="D209" s="77"/>
       <c r="E209" s="27"/>
@@ -8261,8 +8462,8 @@
       <c r="T209" s="27"/>
     </row>
     <row r="210" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A210" s="91"/>
-      <c r="B210" s="80"/>
+      <c r="A210" s="90"/>
+      <c r="B210" s="83"/>
       <c r="C210" s="77"/>
       <c r="D210" s="77"/>
       <c r="E210" s="27"/>
@@ -8283,8 +8484,8 @@
       <c r="T210" s="27"/>
     </row>
     <row r="211" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A211" s="91"/>
-      <c r="B211" s="80"/>
+      <c r="A211" s="90"/>
+      <c r="B211" s="83"/>
       <c r="C211" s="77"/>
       <c r="D211" s="77"/>
       <c r="E211" s="27"/>
@@ -8305,8 +8506,8 @@
       <c r="T211" s="27"/>
     </row>
     <row r="212" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A212" s="91"/>
-      <c r="B212" s="80"/>
+      <c r="A212" s="90"/>
+      <c r="B212" s="83"/>
       <c r="C212" s="77"/>
       <c r="D212" s="77"/>
       <c r="E212" s="27"/>
@@ -8327,8 +8528,8 @@
       <c r="T212" s="27"/>
     </row>
     <row r="213" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A213" s="91"/>
-      <c r="B213" s="80"/>
+      <c r="A213" s="90"/>
+      <c r="B213" s="83"/>
       <c r="C213" s="77"/>
       <c r="D213" s="77"/>
       <c r="E213" s="27"/>
@@ -8349,8 +8550,8 @@
       <c r="T213" s="27"/>
     </row>
     <row r="214" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A214" s="91"/>
-      <c r="B214" s="80"/>
+      <c r="A214" s="90"/>
+      <c r="B214" s="83"/>
       <c r="C214" s="77"/>
       <c r="D214" s="77"/>
       <c r="E214" s="27"/>
@@ -8371,8 +8572,8 @@
       <c r="T214" s="27"/>
     </row>
     <row r="215" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A215" s="91"/>
-      <c r="B215" s="80"/>
+      <c r="A215" s="90"/>
+      <c r="B215" s="83"/>
       <c r="C215" s="77"/>
       <c r="D215" s="77"/>
       <c r="E215" s="27"/>
@@ -8393,8 +8594,8 @@
       <c r="T215" s="27"/>
     </row>
     <row r="216" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A216" s="91"/>
-      <c r="B216" s="80"/>
+      <c r="A216" s="90"/>
+      <c r="B216" s="83"/>
       <c r="C216" s="77"/>
       <c r="D216" s="77"/>
       <c r="E216" s="27"/>
@@ -8415,8 +8616,8 @@
       <c r="T216" s="27"/>
     </row>
     <row r="217" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A217" s="92"/>
-      <c r="B217" s="81"/>
+      <c r="A217" s="91"/>
+      <c r="B217" s="84"/>
       <c r="C217" s="78"/>
       <c r="D217" s="78"/>
       <c r="E217" s="27"/>
@@ -8437,17 +8638,17 @@
       <c r="T217" s="27"/>
     </row>
     <row r="218" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A218" s="90" t="s">
-        <v>231</v>
-      </c>
-      <c r="B218" s="79" t="e" vm="5">
+      <c r="A218" s="89" t="s">
+        <v>255</v>
+      </c>
+      <c r="B218" s="82" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
       <c r="C218" s="76" t="s">
-        <v>232</v>
+        <v>256</v>
       </c>
       <c r="D218" s="76" t="s">
-        <v>233</v>
+        <v>257</v>
       </c>
       <c r="E218" s="27"/>
       <c r="F218" s="27"/>
@@ -8467,8 +8668,8 @@
       <c r="T218" s="27"/>
     </row>
     <row r="219" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A219" s="91"/>
-      <c r="B219" s="80"/>
+      <c r="A219" s="90"/>
+      <c r="B219" s="83"/>
       <c r="C219" s="77"/>
       <c r="D219" s="77"/>
       <c r="E219" s="27"/>
@@ -8489,8 +8690,8 @@
       <c r="T219" s="27"/>
     </row>
     <row r="220" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A220" s="91"/>
-      <c r="B220" s="80"/>
+      <c r="A220" s="90"/>
+      <c r="B220" s="83"/>
       <c r="C220" s="77"/>
       <c r="D220" s="77"/>
       <c r="E220" s="27"/>
@@ -8511,8 +8712,8 @@
       <c r="T220" s="27"/>
     </row>
     <row r="221" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A221" s="91"/>
-      <c r="B221" s="80"/>
+      <c r="A221" s="90"/>
+      <c r="B221" s="83"/>
       <c r="C221" s="77"/>
       <c r="D221" s="77"/>
       <c r="E221" s="27"/>
@@ -8533,8 +8734,8 @@
       <c r="T221" s="27"/>
     </row>
     <row r="222" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A222" s="91"/>
-      <c r="B222" s="80"/>
+      <c r="A222" s="90"/>
+      <c r="B222" s="83"/>
       <c r="C222" s="77"/>
       <c r="D222" s="77"/>
       <c r="E222" s="27"/>
@@ -8555,8 +8756,8 @@
       <c r="T222" s="27"/>
     </row>
     <row r="223" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A223" s="91"/>
-      <c r="B223" s="80"/>
+      <c r="A223" s="90"/>
+      <c r="B223" s="83"/>
       <c r="C223" s="77"/>
       <c r="D223" s="77"/>
       <c r="E223" s="27"/>
@@ -8577,8 +8778,8 @@
       <c r="T223" s="27"/>
     </row>
     <row r="224" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A224" s="91"/>
-      <c r="B224" s="80"/>
+      <c r="A224" s="90"/>
+      <c r="B224" s="83"/>
       <c r="C224" s="77"/>
       <c r="D224" s="77"/>
       <c r="E224" s="27"/>
@@ -8599,8 +8800,8 @@
       <c r="T224" s="27"/>
     </row>
     <row r="225" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A225" s="91"/>
-      <c r="B225" s="80"/>
+      <c r="A225" s="90"/>
+      <c r="B225" s="83"/>
       <c r="C225" s="77"/>
       <c r="D225" s="77"/>
       <c r="E225" s="27"/>
@@ -8621,8 +8822,8 @@
       <c r="T225" s="27"/>
     </row>
     <row r="226" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A226" s="91"/>
-      <c r="B226" s="80"/>
+      <c r="A226" s="90"/>
+      <c r="B226" s="83"/>
       <c r="C226" s="77"/>
       <c r="D226" s="77"/>
       <c r="E226" s="27"/>
@@ -8643,8 +8844,8 @@
       <c r="T226" s="27"/>
     </row>
     <row r="227" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A227" s="91"/>
-      <c r="B227" s="80"/>
+      <c r="A227" s="90"/>
+      <c r="B227" s="83"/>
       <c r="C227" s="77"/>
       <c r="D227" s="77"/>
       <c r="E227" s="27"/>
@@ -8665,8 +8866,8 @@
       <c r="T227" s="27"/>
     </row>
     <row r="228" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A228" s="91"/>
-      <c r="B228" s="80"/>
+      <c r="A228" s="90"/>
+      <c r="B228" s="83"/>
       <c r="C228" s="77"/>
       <c r="D228" s="77"/>
       <c r="E228" s="27"/>
@@ -8687,8 +8888,8 @@
       <c r="T228" s="27"/>
     </row>
     <row r="229" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A229" s="91"/>
-      <c r="B229" s="80"/>
+      <c r="A229" s="90"/>
+      <c r="B229" s="83"/>
       <c r="C229" s="77"/>
       <c r="D229" s="77"/>
       <c r="E229" s="27"/>
@@ -8709,8 +8910,8 @@
       <c r="T229" s="27"/>
     </row>
     <row r="230" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A230" s="91"/>
-      <c r="B230" s="80"/>
+      <c r="A230" s="90"/>
+      <c r="B230" s="83"/>
       <c r="C230" s="77"/>
       <c r="D230" s="77"/>
       <c r="E230" s="27"/>
@@ -8731,8 +8932,8 @@
       <c r="T230" s="27"/>
     </row>
     <row r="231" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A231" s="92"/>
-      <c r="B231" s="81"/>
+      <c r="A231" s="91"/>
+      <c r="B231" s="84"/>
       <c r="C231" s="78"/>
       <c r="D231" s="78"/>
       <c r="E231" s="27"/>
@@ -8753,17 +8954,17 @@
       <c r="T231" s="27"/>
     </row>
     <row r="232" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A232" s="90" t="s">
-        <v>234</v>
-      </c>
-      <c r="B232" s="79" t="e" vm="6">
+      <c r="A232" s="89" t="s">
+        <v>258</v>
+      </c>
+      <c r="B232" s="82" t="e" vm="6">
         <v>#VALUE!</v>
       </c>
       <c r="C232" s="76" t="s">
-        <v>235</v>
+        <v>259</v>
       </c>
       <c r="D232" s="76" t="s">
-        <v>236</v>
+        <v>260</v>
       </c>
       <c r="E232" s="27"/>
       <c r="F232" s="27"/>
@@ -8783,8 +8984,8 @@
       <c r="T232" s="27"/>
     </row>
     <row r="233" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A233" s="91"/>
-      <c r="B233" s="80"/>
+      <c r="A233" s="90"/>
+      <c r="B233" s="83"/>
       <c r="C233" s="77"/>
       <c r="D233" s="77"/>
       <c r="E233" s="27"/>
@@ -8805,8 +9006,8 @@
       <c r="T233" s="27"/>
     </row>
     <row r="234" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A234" s="91"/>
-      <c r="B234" s="80"/>
+      <c r="A234" s="90"/>
+      <c r="B234" s="83"/>
       <c r="C234" s="77"/>
       <c r="D234" s="77"/>
       <c r="E234" s="27"/>
@@ -8827,8 +9028,8 @@
       <c r="T234" s="27"/>
     </row>
     <row r="235" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A235" s="91"/>
-      <c r="B235" s="80"/>
+      <c r="A235" s="90"/>
+      <c r="B235" s="83"/>
       <c r="C235" s="77"/>
       <c r="D235" s="77"/>
       <c r="E235" s="27"/>
@@ -8849,8 +9050,8 @@
       <c r="T235" s="27"/>
     </row>
     <row r="236" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A236" s="91"/>
-      <c r="B236" s="80"/>
+      <c r="A236" s="90"/>
+      <c r="B236" s="83"/>
       <c r="C236" s="77"/>
       <c r="D236" s="77"/>
       <c r="E236" s="27"/>
@@ -8871,8 +9072,8 @@
       <c r="T236" s="27"/>
     </row>
     <row r="237" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A237" s="91"/>
-      <c r="B237" s="80"/>
+      <c r="A237" s="90"/>
+      <c r="B237" s="83"/>
       <c r="C237" s="77"/>
       <c r="D237" s="77"/>
       <c r="E237" s="27"/>
@@ -8893,8 +9094,8 @@
       <c r="T237" s="27"/>
     </row>
     <row r="238" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A238" s="91"/>
-      <c r="B238" s="80"/>
+      <c r="A238" s="90"/>
+      <c r="B238" s="83"/>
       <c r="C238" s="77"/>
       <c r="D238" s="77"/>
       <c r="E238" s="27"/>
@@ -8915,8 +9116,8 @@
       <c r="T238" s="27"/>
     </row>
     <row r="239" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A239" s="91"/>
-      <c r="B239" s="80"/>
+      <c r="A239" s="90"/>
+      <c r="B239" s="83"/>
       <c r="C239" s="77"/>
       <c r="D239" s="77"/>
       <c r="E239" s="27"/>
@@ -8937,8 +9138,8 @@
       <c r="T239" s="27"/>
     </row>
     <row r="240" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A240" s="91"/>
-      <c r="B240" s="80"/>
+      <c r="A240" s="90"/>
+      <c r="B240" s="83"/>
       <c r="C240" s="77"/>
       <c r="D240" s="77"/>
       <c r="E240" s="27"/>
@@ -8959,8 +9160,8 @@
       <c r="T240" s="27"/>
     </row>
     <row r="241" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A241" s="91"/>
-      <c r="B241" s="80"/>
+      <c r="A241" s="90"/>
+      <c r="B241" s="83"/>
       <c r="C241" s="77"/>
       <c r="D241" s="77"/>
       <c r="E241" s="27"/>
@@ -8981,8 +9182,8 @@
       <c r="T241" s="27"/>
     </row>
     <row r="242" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A242" s="91"/>
-      <c r="B242" s="80"/>
+      <c r="A242" s="90"/>
+      <c r="B242" s="83"/>
       <c r="C242" s="77"/>
       <c r="D242" s="77"/>
       <c r="E242" s="27"/>
@@ -9003,8 +9204,8 @@
       <c r="T242" s="27"/>
     </row>
     <row r="243" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A243" s="91"/>
-      <c r="B243" s="80"/>
+      <c r="A243" s="90"/>
+      <c r="B243" s="83"/>
       <c r="C243" s="77"/>
       <c r="D243" s="77"/>
       <c r="E243" s="27"/>
@@ -9025,8 +9226,8 @@
       <c r="T243" s="27"/>
     </row>
     <row r="244" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A244" s="91"/>
-      <c r="B244" s="80"/>
+      <c r="A244" s="90"/>
+      <c r="B244" s="83"/>
       <c r="C244" s="77"/>
       <c r="D244" s="77"/>
       <c r="E244" s="27"/>
@@ -9047,8 +9248,8 @@
       <c r="T244" s="27"/>
     </row>
     <row r="245" spans="1:20" ht="14.45" customHeight="1">
-      <c r="A245" s="92"/>
-      <c r="B245" s="81"/>
+      <c r="A245" s="91"/>
+      <c r="B245" s="84"/>
       <c r="C245" s="78"/>
       <c r="D245" s="78"/>
       <c r="E245" s="27"/>
@@ -9157,10 +9358,10 @@
       <c r="T249" s="27"/>
     </row>
     <row r="250" spans="1:20" ht="15.6" customHeight="1">
-      <c r="A250" s="86" t="s">
-        <v>237</v>
-      </c>
-      <c r="B250" s="86"/>
+      <c r="A250" s="88" t="s">
+        <v>261</v>
+      </c>
+      <c r="B250" s="88"/>
       <c r="C250" s="66"/>
       <c r="D250" s="27"/>
       <c r="E250" s="27"/>
@@ -9204,7 +9405,7 @@
     </row>
     <row r="252" spans="1:20" ht="14.45" customHeight="1">
       <c r="A252" s="29" t="s">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="B252" s="27"/>
       <c r="C252" s="27"/>
@@ -9229,10 +9430,10 @@
     <row r="253" spans="1:20" ht="15.6" customHeight="1">
       <c r="A253" s="66"/>
       <c r="B253" s="67" t="s">
-        <v>238</v>
+        <v>262</v>
       </c>
       <c r="C253" s="68" t="s">
-        <v>239</v>
+        <v>263</v>
       </c>
       <c r="D253" s="27"/>
       <c r="E253" s="27"/>
@@ -9255,10 +9456,10 @@
     <row r="254" spans="1:20" ht="15.6" customHeight="1">
       <c r="A254" s="66"/>
       <c r="B254" s="69" t="s">
-        <v>240</v>
+        <v>264</v>
       </c>
       <c r="C254" s="76" t="s">
-        <v>241</v>
+        <v>265</v>
       </c>
       <c r="D254" s="27"/>
       <c r="E254" s="27"/>
@@ -9281,7 +9482,7 @@
     <row r="255" spans="1:20" ht="15.6" customHeight="1">
       <c r="A255" s="66"/>
       <c r="B255" s="70" t="s">
-        <v>242</v>
+        <v>266</v>
       </c>
       <c r="C255" s="77"/>
       <c r="D255" s="27"/>
@@ -9305,7 +9506,7 @@
     <row r="256" spans="1:20" ht="15.6" customHeight="1">
       <c r="A256" s="66"/>
       <c r="B256" s="71" t="s">
-        <v>243</v>
+        <v>267</v>
       </c>
       <c r="C256" s="77"/>
       <c r="D256" s="27"/>
@@ -9329,7 +9530,7 @@
     <row r="257" spans="1:20" ht="15.6" customHeight="1">
       <c r="A257" s="66"/>
       <c r="B257" s="72" t="s">
-        <v>244</v>
+        <v>268</v>
       </c>
       <c r="C257" s="77"/>
       <c r="D257" s="27"/>
@@ -9353,7 +9554,7 @@
     <row r="258" spans="1:20" ht="62.1" customHeight="1">
       <c r="A258" s="27"/>
       <c r="B258" s="39" t="s">
-        <v>245</v>
+        <v>269</v>
       </c>
       <c r="C258" s="78"/>
       <c r="D258" s="27"/>
@@ -9377,10 +9578,10 @@
     <row r="259" spans="1:20" ht="15.6" customHeight="1">
       <c r="A259" s="27"/>
       <c r="B259" s="72" t="s">
-        <v>246</v>
-      </c>
-      <c r="C259" s="87" t="s">
-        <v>247</v>
+        <v>270</v>
+      </c>
+      <c r="C259" s="85" t="s">
+        <v>271</v>
       </c>
       <c r="D259" s="27"/>
       <c r="E259" s="27"/>
@@ -9403,9 +9604,9 @@
     <row r="260" spans="1:20" ht="15" customHeight="1">
       <c r="A260" s="27"/>
       <c r="B260" s="73" t="s">
-        <v>248</v>
-      </c>
-      <c r="C260" s="88"/>
+        <v>272</v>
+      </c>
+      <c r="C260" s="86"/>
       <c r="D260" s="27"/>
       <c r="E260" s="27"/>
       <c r="F260" s="27"/>
@@ -9427,7 +9628,7 @@
     <row r="261" spans="1:20" ht="15.6" customHeight="1">
       <c r="A261" s="27"/>
       <c r="B261" s="74"/>
-      <c r="C261" s="88"/>
+      <c r="C261" s="86"/>
       <c r="D261" s="27"/>
       <c r="E261" s="27"/>
       <c r="F261" s="27"/>
@@ -9449,7 +9650,7 @@
     <row r="262" spans="1:20" ht="15.6" customHeight="1">
       <c r="A262" s="27"/>
       <c r="B262" s="74"/>
-      <c r="C262" s="89"/>
+      <c r="C262" s="87"/>
       <c r="D262" s="27"/>
       <c r="E262" s="27"/>
       <c r="F262" s="27"/>
@@ -9471,10 +9672,10 @@
     <row r="263" spans="1:20" ht="15.6" customHeight="1">
       <c r="A263" s="27"/>
       <c r="B263" s="72" t="s">
-        <v>249</v>
-      </c>
-      <c r="C263" s="87" t="s">
-        <v>250</v>
+        <v>273</v>
+      </c>
+      <c r="C263" s="85" t="s">
+        <v>274</v>
       </c>
       <c r="D263" s="27"/>
       <c r="E263" s="27"/>
@@ -9497,7 +9698,7 @@
     <row r="264" spans="1:20" ht="15.6" customHeight="1">
       <c r="A264" s="27"/>
       <c r="B264" s="74"/>
-      <c r="C264" s="88"/>
+      <c r="C264" s="86"/>
       <c r="D264" s="27"/>
       <c r="E264" s="27"/>
       <c r="F264" s="27"/>
@@ -9519,7 +9720,7 @@
     <row r="265" spans="1:20" ht="15.6" customHeight="1">
       <c r="A265" s="27"/>
       <c r="B265" s="74"/>
-      <c r="C265" s="89"/>
+      <c r="C265" s="87"/>
       <c r="D265" s="27"/>
       <c r="E265" s="27"/>
       <c r="F265" s="27"/>
@@ -9541,10 +9742,10 @@
     <row r="266" spans="1:20" ht="15.6" customHeight="1">
       <c r="A266" s="27"/>
       <c r="B266" s="72" t="s">
-        <v>251</v>
+        <v>275</v>
       </c>
       <c r="C266" s="76" t="s">
-        <v>252</v>
+        <v>276</v>
       </c>
       <c r="D266" s="27"/>
       <c r="E266" s="27"/>
@@ -9611,7 +9812,7 @@
     <row r="269" spans="1:20" ht="30.95" customHeight="1">
       <c r="A269" s="27"/>
       <c r="B269" s="39" t="s">
-        <v>253</v>
+        <v>277</v>
       </c>
       <c r="C269" s="78"/>
       <c r="D269" s="27"/>
@@ -9635,10 +9836,10 @@
     <row r="270" spans="1:20" ht="15" customHeight="1">
       <c r="A270" s="27"/>
       <c r="B270" s="71" t="s">
-        <v>254</v>
+        <v>278</v>
       </c>
       <c r="C270" s="76" t="s">
-        <v>255</v>
+        <v>279</v>
       </c>
       <c r="D270" s="27"/>
       <c r="E270" s="27"/>
@@ -9661,7 +9862,7 @@
     <row r="271" spans="1:20" ht="15" customHeight="1">
       <c r="A271" s="27"/>
       <c r="B271" s="71" t="s">
-        <v>148</v>
+        <v>172</v>
       </c>
       <c r="C271" s="77"/>
       <c r="D271" s="27"/>
@@ -9685,7 +9886,7 @@
     <row r="272" spans="1:20" ht="15.6" customHeight="1">
       <c r="A272" s="27"/>
       <c r="B272" s="72" t="s">
-        <v>256</v>
+        <v>280</v>
       </c>
       <c r="C272" s="77"/>
       <c r="D272" s="27"/>
@@ -9709,7 +9910,7 @@
     <row r="273" spans="1:20" ht="46.5" customHeight="1">
       <c r="A273" s="27"/>
       <c r="B273" s="39" t="s">
-        <v>257</v>
+        <v>281</v>
       </c>
       <c r="C273" s="77"/>
       <c r="D273" s="27"/>
@@ -9733,7 +9934,7 @@
     <row r="274" spans="1:20" ht="15.6" customHeight="1">
       <c r="A274" s="27"/>
       <c r="B274" s="71" t="s">
-        <v>258</v>
+        <v>282</v>
       </c>
       <c r="C274" s="77"/>
       <c r="D274" s="27"/>
@@ -9757,7 +9958,7 @@
     <row r="275" spans="1:20" ht="15.6" customHeight="1">
       <c r="A275" s="27"/>
       <c r="B275" s="71" t="s">
-        <v>259</v>
+        <v>283</v>
       </c>
       <c r="C275" s="77"/>
       <c r="D275" s="27"/>
@@ -9781,7 +9982,7 @@
     <row r="276" spans="1:20" ht="15" customHeight="1">
       <c r="A276" s="27"/>
       <c r="B276" s="71" t="s">
-        <v>260</v>
+        <v>284</v>
       </c>
       <c r="C276" s="77"/>
       <c r="D276" s="27"/>
@@ -9805,7 +10006,7 @@
     <row r="277" spans="1:20" ht="15" customHeight="1">
       <c r="A277" s="27"/>
       <c r="B277" s="71" t="s">
-        <v>261</v>
+        <v>285</v>
       </c>
       <c r="C277" s="78"/>
       <c r="D277" s="27"/>
@@ -9829,10 +10030,10 @@
     <row r="278" spans="1:20" ht="15" customHeight="1">
       <c r="A278" s="27"/>
       <c r="B278" s="71" t="s">
-        <v>262</v>
+        <v>286</v>
       </c>
       <c r="C278" s="76" t="s">
-        <v>263</v>
+        <v>287</v>
       </c>
       <c r="D278" s="27"/>
       <c r="E278" s="27"/>
@@ -9855,7 +10056,7 @@
     <row r="279" spans="1:20" ht="15.6" customHeight="1">
       <c r="A279" s="27"/>
       <c r="B279" s="72" t="s">
-        <v>264</v>
+        <v>288</v>
       </c>
       <c r="C279" s="77"/>
       <c r="D279" s="27"/>
@@ -9879,7 +10080,7 @@
     <row r="280" spans="1:20" ht="46.5" customHeight="1">
       <c r="A280" s="27"/>
       <c r="B280" s="39" t="s">
-        <v>265</v>
+        <v>289</v>
       </c>
       <c r="C280" s="77"/>
       <c r="D280" s="27"/>
@@ -9903,7 +10104,7 @@
     <row r="281" spans="1:20" ht="15.6" customHeight="1">
       <c r="A281" s="27"/>
       <c r="B281" s="71" t="s">
-        <v>266</v>
+        <v>290</v>
       </c>
       <c r="C281" s="77"/>
       <c r="D281" s="27"/>
@@ -9927,7 +10128,7 @@
     <row r="282" spans="1:20" ht="15.6" customHeight="1">
       <c r="A282" s="27"/>
       <c r="B282" s="71" t="s">
-        <v>259</v>
+        <v>283</v>
       </c>
       <c r="C282" s="77"/>
       <c r="D282" s="27"/>
@@ -9951,7 +10152,7 @@
     <row r="283" spans="1:20" ht="15" customHeight="1">
       <c r="A283" s="27"/>
       <c r="B283" s="71" t="s">
-        <v>260</v>
+        <v>284</v>
       </c>
       <c r="C283" s="77"/>
       <c r="D283" s="27"/>
@@ -9975,7 +10176,7 @@
     <row r="284" spans="1:20" ht="15" customHeight="1">
       <c r="A284" s="27"/>
       <c r="B284" s="75" t="s">
-        <v>261</v>
+        <v>285</v>
       </c>
       <c r="C284" s="78"/>
       <c r="D284" s="27"/>
@@ -10021,6 +10222,35 @@
     <row r="286" spans="1:20" ht="15"/>
   </sheetData>
   <mergeCells count="45">
+    <mergeCell ref="C232:C245"/>
+    <mergeCell ref="B162:B175"/>
+    <mergeCell ref="D162:D175"/>
+    <mergeCell ref="C266:C269"/>
+    <mergeCell ref="A29:A31"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A250:B250"/>
+    <mergeCell ref="C259:C262"/>
+    <mergeCell ref="D176:D189"/>
+    <mergeCell ref="D232:D245"/>
+    <mergeCell ref="D190:D203"/>
+    <mergeCell ref="A232:A245"/>
+    <mergeCell ref="D218:D231"/>
+    <mergeCell ref="D204:D217"/>
+    <mergeCell ref="A218:A231"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A190:A203"/>
+    <mergeCell ref="A18:A24"/>
+    <mergeCell ref="C190:C203"/>
+    <mergeCell ref="B204:B217"/>
+    <mergeCell ref="B12:B17"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="A176:A189"/>
+    <mergeCell ref="A12:A17"/>
+    <mergeCell ref="A162:A175"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="B18:B24"/>
+    <mergeCell ref="A25:A27"/>
+    <mergeCell ref="B9:B11"/>
     <mergeCell ref="C278:C284"/>
     <mergeCell ref="C254:C258"/>
     <mergeCell ref="B25:B27"/>
@@ -10037,233 +10267,6 @@
     <mergeCell ref="A111:B111"/>
     <mergeCell ref="A204:A217"/>
     <mergeCell ref="C176:C189"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A190:A203"/>
-    <mergeCell ref="A18:A24"/>
-    <mergeCell ref="C190:C203"/>
-    <mergeCell ref="B204:B217"/>
-    <mergeCell ref="B12:B17"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="A176:A189"/>
-    <mergeCell ref="A12:A17"/>
-    <mergeCell ref="A162:A175"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="B18:B24"/>
-    <mergeCell ref="A25:A27"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="C232:C245"/>
-    <mergeCell ref="B162:B175"/>
-    <mergeCell ref="D162:D175"/>
-    <mergeCell ref="C266:C269"/>
-    <mergeCell ref="A29:A31"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A250:B250"/>
-    <mergeCell ref="C259:C262"/>
-    <mergeCell ref="D176:D189"/>
-    <mergeCell ref="D232:D245"/>
-    <mergeCell ref="D190:D203"/>
-    <mergeCell ref="A232:A245"/>
-    <mergeCell ref="D218:D231"/>
-    <mergeCell ref="D204:D217"/>
-    <mergeCell ref="A218:A231"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C29"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
-  <cols>
-    <col min="1" max="1" width="18.5703125" customWidth="1"/>
-    <col min="2" max="2" width="86.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="101" t="s">
-        <v>267</v>
-      </c>
-      <c r="B1" s="104"/>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="104"/>
-      <c r="B2" s="104"/>
-    </row>
-    <row r="4" spans="1:3" ht="15" customHeight="1" thickBot="1"/>
-    <row r="5" spans="1:3" ht="15.6" customHeight="1" thickBot="1">
-      <c r="A5" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="126" customHeight="1" thickBot="1">
-      <c r="A6" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="15" customHeight="1">
-      <c r="A7" s="102" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>270</v>
-      </c>
-      <c r="C7" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="15" customHeight="1">
-      <c r="A8" s="105"/>
-      <c r="B8" s="5" t="s">
-        <v>272</v>
-      </c>
-      <c r="C8" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="15.6" customHeight="1" thickBot="1">
-      <c r="A9" s="106"/>
-      <c r="B9" s="6" t="s">
-        <v>274</v>
-      </c>
-      <c r="C9" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="30.75">
-      <c r="A10" s="102" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="61.5">
-      <c r="A11" s="105"/>
-      <c r="B11" s="8" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="30.75">
-      <c r="A12" s="105"/>
-      <c r="B12" s="8" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="30.75">
-      <c r="A13" s="105"/>
-      <c r="B13" s="8" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="30.75">
-      <c r="A14" s="105"/>
-      <c r="B14" s="8" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="30.75" thickBot="1">
-      <c r="A15" s="106"/>
-      <c r="B15" s="9" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="30.75">
-      <c r="A16" s="102" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="30.75">
-      <c r="A17" s="105"/>
-      <c r="B17" s="8" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="30.75">
-      <c r="A18" s="105"/>
-      <c r="B18" s="8" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="30.75">
-      <c r="A19" s="105"/>
-      <c r="B19" s="8" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="15.6" customHeight="1">
-      <c r="A20" s="105"/>
-      <c r="B20" s="8"/>
-    </row>
-    <row r="21" spans="1:2" ht="15.6" customHeight="1">
-      <c r="A21" s="105"/>
-      <c r="B21" s="8"/>
-    </row>
-    <row r="22" spans="1:2" ht="15.95" customHeight="1" thickBot="1">
-      <c r="A22" s="106"/>
-      <c r="B22" s="9"/>
-    </row>
-    <row r="23" spans="1:2" ht="30.75">
-      <c r="A23" s="102" t="s">
-        <v>31</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="30.75">
-      <c r="A24" s="105"/>
-      <c r="B24" s="8" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="30.75" thickBot="1">
-      <c r="A25" s="106"/>
-      <c r="B25" s="9" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="30.6" customHeight="1" thickBot="1">
-      <c r="A26" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="15.6" customHeight="1">
-      <c r="A27" s="102" t="s">
-        <v>39</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="15.6" customHeight="1">
-      <c r="A28" s="105"/>
-      <c r="B28" s="8"/>
-    </row>
-    <row r="29" spans="1:2" ht="15.95" customHeight="1" thickBot="1">
-      <c r="A29" s="106"/>
-      <c r="B29" s="9"/>
-    </row>
-  </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A1:B2"/>
-    <mergeCell ref="A27:A29"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="A16:A22"/>
-    <mergeCell ref="A10:A15"/>
-    <mergeCell ref="A23:A25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10293,19 +10296,19 @@
         <v>291</v>
       </c>
       <c r="B1" s="23" t="s">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="C1" s="23" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
       <c r="D1" s="23" t="s">
         <v>292</v>
       </c>
       <c r="E1" s="23" t="s">
-        <v>51</v>
+        <v>75</v>
       </c>
       <c r="F1" s="23" t="s">
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="G1" s="23" t="s">
         <v>293</v>
@@ -10317,22 +10320,22 @@
         <v>295</v>
       </c>
       <c r="J1" s="24" t="s">
-        <v>55</v>
+        <v>79</v>
       </c>
       <c r="K1" s="25" t="s">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="L1" s="24" t="s">
-        <v>57</v>
+        <v>81</v>
       </c>
       <c r="M1" s="24" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="N1" s="25" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="O1" s="25" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="P1" s="25" t="s">
         <v>296</v>
@@ -10341,37 +10344,37 @@
         <v>297</v>
       </c>
       <c r="R1" s="23" t="s">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="S1" s="23" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="T1" s="23" t="s">
-        <v>71</v>
+        <v>95</v>
       </c>
       <c r="U1" s="23" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="V1" s="23" t="s">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="W1" s="23" t="s">
         <v>298</v>
       </c>
       <c r="X1" s="23" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
       <c r="Y1" s="23" t="s">
-        <v>81</v>
+        <v>105</v>
       </c>
       <c r="Z1" s="23" t="s">
-        <v>83</v>
+        <v>107</v>
       </c>
       <c r="AA1" s="23" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="AB1" s="26" t="s">
-        <v>89</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:28" ht="14.1" customHeight="1">
@@ -11191,57 +11194,57 @@
   <sheetData>
     <row r="1" spans="1:18" s="2" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>119</v>
+        <v>143</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>122</v>
+        <v>146</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>127</v>
+        <v>151</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>133</v>
+        <v>157</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>136</v>
+        <v>160</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>142</v>
+        <v>166</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>145</v>
+        <v>169</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>148</v>
+        <v>172</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>151</v>
+        <v>175</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>358</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>160</v>
+        <v>184</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>163</v>
+        <v>187</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>166</v>
+        <v>190</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>169</v>
+        <v>193</v>
       </c>
       <c r="Q1" s="103" t="s">
-        <v>172</v>
-      </c>
-      <c r="R1" s="107"/>
+        <v>196</v>
+      </c>
+      <c r="R1" s="108"/>
     </row>
     <row r="2" spans="1:18">
       <c r="A2" t="s">
@@ -11363,6 +11366,7 @@
   <cols>
     <col min="1" max="1" width="38.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="94" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35" customWidth="1"/>
     <col min="6" max="6" width="6.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="30.5703125" bestFit="1" customWidth="1"/>
@@ -11379,63 +11383,63 @@
     <col min="19" max="19" width="52.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="22" customFormat="1" ht="15.95" customHeight="1">
-      <c r="A1" s="22" t="s">
-        <v>176</v>
-      </c>
-      <c r="B1" s="22" t="s">
-        <v>177</v>
-      </c>
-      <c r="C1" s="22" t="s">
-        <v>178</v>
-      </c>
-      <c r="D1" s="22" t="s">
-        <v>179</v>
-      </c>
-      <c r="E1" s="22" t="s">
-        <v>180</v>
-      </c>
-      <c r="F1" s="22" t="s">
-        <v>181</v>
-      </c>
-      <c r="G1" s="22" t="s">
-        <v>182</v>
-      </c>
-      <c r="H1" s="22" t="s">
-        <v>183</v>
-      </c>
-      <c r="I1" s="22" t="s">
-        <v>184</v>
-      </c>
-      <c r="J1" s="22" t="s">
-        <v>185</v>
-      </c>
-      <c r="K1" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="L1" s="22" t="s">
-        <v>186</v>
-      </c>
-      <c r="M1" s="22" t="s">
-        <v>187</v>
-      </c>
-      <c r="N1" s="22" t="s">
-        <v>188</v>
-      </c>
-      <c r="O1" s="22" t="s">
-        <v>189</v>
-      </c>
-      <c r="P1" s="22" t="s">
-        <v>190</v>
-      </c>
-      <c r="Q1" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="R1" s="22" t="s">
-        <v>192</v>
-      </c>
-      <c r="S1" s="22" t="s">
-        <v>193</v>
+    <row r="1" spans="1:19" s="104" customFormat="1" ht="53.25" customHeight="1">
+      <c r="A1" s="104" t="s">
+        <v>200</v>
+      </c>
+      <c r="B1" s="104" t="s">
+        <v>201</v>
+      </c>
+      <c r="C1" s="104" t="s">
+        <v>202</v>
+      </c>
+      <c r="D1" s="104" t="s">
+        <v>203</v>
+      </c>
+      <c r="E1" s="104" t="s">
+        <v>204</v>
+      </c>
+      <c r="F1" s="104" t="s">
+        <v>205</v>
+      </c>
+      <c r="G1" s="104" t="s">
+        <v>206</v>
+      </c>
+      <c r="H1" s="104" t="s">
+        <v>207</v>
+      </c>
+      <c r="I1" s="104" t="s">
+        <v>208</v>
+      </c>
+      <c r="J1" s="104" t="s">
+        <v>209</v>
+      </c>
+      <c r="K1" s="104" t="s">
+        <v>101</v>
+      </c>
+      <c r="L1" s="104" t="s">
+        <v>210</v>
+      </c>
+      <c r="M1" s="104" t="s">
+        <v>211</v>
+      </c>
+      <c r="N1" s="104" t="s">
+        <v>212</v>
+      </c>
+      <c r="O1" s="104" t="s">
+        <v>213</v>
+      </c>
+      <c r="P1" s="104" t="s">
+        <v>214</v>
+      </c>
+      <c r="Q1" s="104" t="s">
+        <v>215</v>
+      </c>
+      <c r="R1" s="104" t="s">
+        <v>216</v>
+      </c>
+      <c r="S1" s="104" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="2" spans="1:19">
@@ -11461,7 +11465,7 @@
         <v>302</v>
       </c>
       <c r="I2" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="J2" t="s">
         <v>326</v>
@@ -11493,7 +11497,7 @@
         <v>302</v>
       </c>
       <c r="I3" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="J3" t="s">
         <v>303</v>
@@ -11525,7 +11529,7 @@
         <v>302</v>
       </c>
       <c r="I4" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="J4" t="s">
         <v>313</v>
@@ -11557,7 +11561,7 @@
         <v>338</v>
       </c>
       <c r="I5" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="J5" t="s">
         <v>326</v>
@@ -11589,7 +11593,7 @@
         <v>338</v>
       </c>
       <c r="I6" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="J6" t="s">
         <v>303</v>
@@ -11621,7 +11625,7 @@
         <v>338</v>
       </c>
       <c r="I7" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="J7" t="s">
         <v>341</v>
@@ -11653,7 +11657,7 @@
         <v>338</v>
       </c>
       <c r="I8" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="J8" t="s">
         <v>343</v>
@@ -11685,7 +11689,7 @@
         <v>349</v>
       </c>
       <c r="I9" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="J9" t="s">
         <v>326</v>
@@ -11717,7 +11721,7 @@
         <v>349</v>
       </c>
       <c r="I10" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="J10" t="s">
         <v>303</v>
@@ -11749,7 +11753,7 @@
         <v>349</v>
       </c>
       <c r="I11" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="J11" t="s">
         <v>341</v>
@@ -11781,7 +11785,7 @@
         <v>349</v>
       </c>
       <c r="I12" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="J12" t="s">
         <v>343</v>
@@ -11813,7 +11817,7 @@
         <v>350</v>
       </c>
       <c r="I13" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="J13" t="s">
         <v>326</v>
@@ -11845,7 +11849,7 @@
         <v>350</v>
       </c>
       <c r="I14" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="J14" t="s">
         <v>353</v>
@@ -11877,7 +11881,7 @@
         <v>350</v>
       </c>
       <c r="I15" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
       <c r="J15" t="s">
         <v>341</v>
@@ -11905,7 +11909,7 @@
   <sheetData>
     <row r="2" spans="2:14">
       <c r="B2" s="20" t="s">
-        <v>216</v>
+        <v>240</v>
       </c>
       <c r="C2" s="20" t="s">
         <v>418</v>
@@ -11952,12 +11956,12 @@
   <sheetData>
     <row r="3" spans="1:1" ht="15" customHeight="1">
       <c r="A3" s="12" t="s">
-        <v>240</v>
+        <v>264</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="15" customHeight="1">
       <c r="A4" s="13" t="s">
-        <v>242</v>
+        <v>266</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="15.6" customHeight="1">
@@ -11967,7 +11971,7 @@
     </row>
     <row r="6" spans="1:1" ht="21" customHeight="1">
       <c r="A6" s="15" t="s">
-        <v>244</v>
+        <v>268</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="21.75" customHeight="1">
@@ -11980,12 +11984,12 @@
     </row>
     <row r="9" spans="1:1" ht="15.6" customHeight="1">
       <c r="A9" s="15" t="s">
-        <v>246</v>
+        <v>270</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="15" customHeight="1">
       <c r="A10" s="16" t="s">
-        <v>248</v>
+        <v>272</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="15.6" customHeight="1">
@@ -12018,27 +12022,27 @@
     </row>
     <row r="19" spans="1:1" ht="30.95" customHeight="1">
       <c r="A19" s="11" t="s">
-        <v>253</v>
+        <v>277</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="15" customHeight="1">
       <c r="A20" s="14" t="s">
-        <v>254</v>
+        <v>278</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="15" customHeight="1">
       <c r="A21" s="14" t="s">
-        <v>148</v>
+        <v>172</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="15.6" customHeight="1">
       <c r="A22" s="15" t="s">
-        <v>256</v>
+        <v>280</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="46.5" customHeight="1">
       <c r="A23" s="11" t="s">
-        <v>257</v>
+        <v>281</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="15.6" customHeight="1">
@@ -12053,27 +12057,27 @@
     </row>
     <row r="26" spans="1:1" ht="15" customHeight="1">
       <c r="A26" s="14" t="s">
-        <v>260</v>
+        <v>284</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="15" customHeight="1">
       <c r="A27" s="14" t="s">
-        <v>261</v>
+        <v>285</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="15" customHeight="1">
       <c r="A28" s="14" t="s">
-        <v>262</v>
+        <v>286</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="15.6" customHeight="1">
       <c r="A29" s="15" t="s">
-        <v>264</v>
+        <v>288</v>
       </c>
     </row>
     <row r="30" spans="1:1" ht="46.5" customHeight="1">
       <c r="A30" s="11" t="s">
-        <v>265</v>
+        <v>289</v>
       </c>
     </row>
     <row r="31" spans="1:1" ht="15.6" customHeight="1">
@@ -12088,12 +12092,12 @@
     </row>
     <row r="33" spans="1:1" ht="15" customHeight="1">
       <c r="A33" s="14" t="s">
-        <v>260</v>
+        <v>284</v>
       </c>
     </row>
     <row r="34" spans="1:1" ht="15" customHeight="1">
       <c r="A34" s="18" t="s">
-        <v>261</v>
+        <v>285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>